<commit_message>
Add daily sales wizard with shop reporting and Excel export
- DailySale model with shop (Fig Tree, Empire Shop, Emirates, Small City), decimal quantities and per-sale cost price
- Daily sales wizard: shop picker, one card per product, manual custom entries, auto-calculated profit
- All-shops daily report page + Excel export with per-shop totals and grand total
- Enable DEBUG by default and harden date/session handling to prevent 500s
- Import command to seed products/transactions from Excel source files
</commit_message>
<xml_diff>
--- a/price list.xlsx
+++ b/price list.xlsx
@@ -1,42 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Downloads\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCBA91E9-674F-4B52-AA9F-C094D6C5E89C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0A905285-55EE-4227-A461-042B81A3081E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
   </bookViews>
   <sheets>
-    <sheet name="all" sheetId="2" r:id="rId1"/>
+    <sheet sheetId="2" name="all" state="visible" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="110">
   <si>
     <t>Product</t>
   </si>
@@ -44,12 +22,24 @@
     <t>Cost Price</t>
   </si>
   <si>
+    <t>Selling Price</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
     <t>Gilbeys</t>
   </si>
   <si>
+    <t>250ml</t>
+  </si>
+  <si>
     <t>Best Whiskey</t>
   </si>
   <si>
+    <t/>
+  </si>
+  <si>
     <t xml:space="preserve">Blue Ice </t>
   </si>
   <si>
@@ -152,6 +142,9 @@
     <t xml:space="preserve"> </t>
   </si>
   <si>
+    <t>350ml</t>
+  </si>
+  <si>
     <t>Black&amp;white</t>
   </si>
   <si>
@@ -161,9 +154,15 @@
     <t>Viceroy</t>
   </si>
   <si>
+    <t>375ml</t>
+  </si>
+  <si>
     <t>VAT 69</t>
   </si>
   <si>
+    <t>750ml</t>
+  </si>
+  <si>
     <t>Brand 750ml</t>
   </si>
   <si>
@@ -191,6 +190,9 @@
     <t>William Lawsons</t>
   </si>
   <si>
+    <t>1200</t>
+  </si>
+  <si>
     <t>Amarula 1ltr</t>
   </si>
   <si>
@@ -230,6 +232,9 @@
     <t xml:space="preserve">Guarana </t>
   </si>
   <si>
+    <t>cans</t>
+  </si>
+  <si>
     <t>Guarana Black</t>
   </si>
   <si>
@@ -266,6 +271,9 @@
     <t>Balozi</t>
   </si>
   <si>
+    <t>Whitecup</t>
+  </si>
+  <si>
     <t>Caprice</t>
   </si>
   <si>
@@ -281,6 +289,12 @@
     <t xml:space="preserve">Pilsner </t>
   </si>
   <si>
+    <t>White Cup Bottle</t>
+  </si>
+  <si>
+    <t>soda</t>
+  </si>
+  <si>
     <t xml:space="preserve">Kingfisher </t>
   </si>
   <si>
@@ -330,80 +344,50 @@
   </si>
   <si>
     <t>Glacier Big</t>
-  </si>
-  <si>
-    <t>Category</t>
-  </si>
-  <si>
-    <t>250ml</t>
-  </si>
-  <si>
-    <t>350ml</t>
-  </si>
-  <si>
-    <t>750ml</t>
-  </si>
-  <si>
-    <t>cans</t>
-  </si>
-  <si>
-    <t>soda</t>
-  </si>
-  <si>
-    <t>Selling Price</t>
-  </si>
-  <si>
-    <t>375ml</t>
-  </si>
-  <si>
-    <t>Whitecup</t>
-  </si>
-  <si>
-    <t>White Cup Bottle</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="5" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <sz val="16"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="16"/>
+      <name val="Aptos Narrow"/>
     </font>
     <font>
       <b/>
-      <sz val="14"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="14"/>
+      <name val="Aptos Narrow"/>
     </font>
     <font>
       <b/>
-      <sz val="17"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="17"/>
+      <name val="Aptos Narrow"/>
     </font>
     <font>
       <b/>
+      <color theme="1"/>
+      <family val="2"/>
       <sz val="14"/>
-      <color theme="1"/>
       <name val="Arial Black"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -430,10 +414,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -767,17 +751,17 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21C1493C-5078-47B4-B77C-A9C8A0DC9D89}">
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D122"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="18" customWidth="1"/>
     <col min="3" max="3" width="19.5703125" customWidth="1"/>
     <col min="4" max="4" width="25.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="22.5" x14ac:dyDescent="0.35">
+    <row r="1" ht="22.5" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -785,15 +769,15 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>98</v>
+        <v>2</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B2">
         <v>416</v>
@@ -802,26 +786,26 @@
         <v>550</v>
       </c>
       <c r="D2" t="s">
-        <v>99</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3">
-        <v>300</v>
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>7</v>
       </c>
       <c r="C3">
         <v>450</v>
       </c>
       <c r="D3" t="s">
-        <v>99</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="B4">
         <v>150</v>
@@ -830,12 +814,12 @@
         <v>160</v>
       </c>
       <c r="D4" t="s">
-        <v>99</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="B5">
         <v>295</v>
@@ -844,26 +828,26 @@
         <v>300</v>
       </c>
       <c r="D5" t="s">
-        <v>99</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6">
-        <v>190</v>
+        <v>10</v>
+      </c>
+      <c r="B6" t="s">
+        <v>7</v>
       </c>
       <c r="C6">
         <v>550</v>
       </c>
       <c r="D6" t="s">
-        <v>99</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="B7">
         <v>395</v>
@@ -872,23 +856,23 @@
         <v>550</v>
       </c>
       <c r="D7" t="s">
-        <v>99</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C8">
         <v>500</v>
       </c>
       <c r="D8" t="s">
-        <v>99</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B9">
         <v>195</v>
@@ -897,23 +881,23 @@
         <v>300</v>
       </c>
       <c r="D9" t="s">
-        <v>99</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="C10">
         <v>300</v>
       </c>
       <c r="D10" t="s">
-        <v>99</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B11">
         <v>225</v>
@@ -922,23 +906,23 @@
         <v>300</v>
       </c>
       <c r="D11" t="s">
-        <v>99</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="C12">
         <v>550</v>
       </c>
       <c r="D12" t="s">
-        <v>99</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B13">
         <v>95</v>
@@ -947,12 +931,12 @@
         <v>200</v>
       </c>
       <c r="D13" t="s">
-        <v>99</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="B14">
         <v>340</v>
@@ -961,12 +945,12 @@
         <v>450</v>
       </c>
       <c r="D14" t="s">
-        <v>99</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="B15">
         <v>334</v>
@@ -975,12 +959,12 @@
         <v>400</v>
       </c>
       <c r="D15" t="s">
-        <v>99</v>
+        <v>5</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="B16">
         <v>232</v>
@@ -989,12 +973,12 @@
         <v>300</v>
       </c>
       <c r="D16" t="s">
-        <v>99</v>
+        <v>5</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B17">
         <v>208</v>
@@ -1003,12 +987,12 @@
         <v>300</v>
       </c>
       <c r="D17" t="s">
-        <v>99</v>
+        <v>5</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="B18">
         <v>197</v>
@@ -1017,12 +1001,12 @@
         <v>300</v>
       </c>
       <c r="D18" t="s">
-        <v>99</v>
+        <v>5</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B19">
         <v>225</v>
@@ -1031,12 +1015,12 @@
         <v>300</v>
       </c>
       <c r="D19" t="s">
-        <v>99</v>
+        <v>5</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="B20">
         <v>285</v>
@@ -1045,26 +1029,26 @@
         <v>400</v>
       </c>
       <c r="D20" t="s">
-        <v>99</v>
+        <v>5</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>21</v>
-      </c>
-      <c r="B21">
-        <v>285</v>
+        <v>25</v>
+      </c>
+      <c r="B21" t="s">
+        <v>7</v>
       </c>
       <c r="C21">
         <v>400</v>
       </c>
       <c r="D21" t="s">
-        <v>99</v>
+        <v>5</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="B22">
         <v>200</v>
@@ -1073,23 +1057,23 @@
         <v>300</v>
       </c>
       <c r="D22" t="s">
-        <v>99</v>
+        <v>5</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="C23">
         <v>600</v>
       </c>
       <c r="D23" t="s">
-        <v>99</v>
+        <v>5</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="B24">
         <v>210</v>
@@ -1098,12 +1082,12 @@
         <v>300</v>
       </c>
       <c r="D24" t="s">
-        <v>99</v>
+        <v>5</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B25">
         <v>125</v>
@@ -1112,12 +1096,12 @@
         <v>160</v>
       </c>
       <c r="D25" t="s">
-        <v>99</v>
+        <v>5</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="B26">
         <v>100</v>
@@ -1126,12 +1110,12 @@
         <v>160</v>
       </c>
       <c r="D26" t="s">
-        <v>99</v>
+        <v>5</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B27">
         <v>285</v>
@@ -1140,12 +1124,12 @@
         <v>400</v>
       </c>
       <c r="D27" t="s">
-        <v>99</v>
+        <v>5</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="B28">
         <v>210</v>
@@ -1154,12 +1138,12 @@
         <v>300</v>
       </c>
       <c r="D28" t="s">
-        <v>99</v>
+        <v>5</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="B29">
         <v>231</v>
@@ -1168,12 +1152,12 @@
         <v>300</v>
       </c>
       <c r="D29" t="s">
-        <v>99</v>
+        <v>5</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B30">
         <v>200</v>
@@ -1182,12 +1166,12 @@
         <v>300</v>
       </c>
       <c r="D30" t="s">
-        <v>99</v>
+        <v>5</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B31">
         <v>95</v>
@@ -1196,12 +1180,12 @@
         <v>160</v>
       </c>
       <c r="D31" t="s">
-        <v>99</v>
+        <v>5</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="B32">
         <v>256</v>
@@ -1210,12 +1194,12 @@
         <v>330</v>
       </c>
       <c r="D32" t="s">
-        <v>99</v>
+        <v>5</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="B33">
         <v>256</v>
@@ -1224,12 +1208,12 @@
         <v>330</v>
       </c>
       <c r="D33" t="s">
-        <v>99</v>
+        <v>5</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="B34">
         <v>256</v>
@@ -1238,54 +1222,54 @@
         <v>330</v>
       </c>
       <c r="D34" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A35" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="B35" s="3"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="35" ht="18.75" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B35" s="4"/>
       <c r="D35" t="s">
-        <v>100</v>
+        <v>7</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C36" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="D36" t="s">
-        <v>100</v>
+        <v>42</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="C37">
         <v>800</v>
       </c>
       <c r="D37" t="s">
-        <v>100</v>
+        <v>42</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="C38">
         <v>1100</v>
       </c>
       <c r="D38" t="s">
-        <v>100</v>
+        <v>42</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B39">
         <v>580</v>
@@ -1294,56 +1278,56 @@
         <v>850</v>
       </c>
       <c r="D39" t="s">
-        <v>100</v>
+        <v>42</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C40">
         <v>850</v>
       </c>
       <c r="D40" t="s">
-        <v>100</v>
+        <v>42</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="C41">
         <v>500</v>
       </c>
       <c r="D41" t="s">
-        <v>100</v>
+        <v>42</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="C42">
         <v>550</v>
       </c>
       <c r="D42" t="s">
-        <v>100</v>
+        <v>42</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C43">
         <v>750</v>
       </c>
       <c r="D43" t="s">
-        <v>100</v>
+        <v>42</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="B44">
         <v>575</v>
@@ -1352,32 +1336,32 @@
         <v>800</v>
       </c>
       <c r="D44" t="s">
-        <v>105</v>
+        <v>46</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="C45">
         <v>800</v>
       </c>
       <c r="D45" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" ht="22.5" x14ac:dyDescent="0.35">
-      <c r="A46" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="B46" s="4"/>
+        <v>48</v>
+      </c>
+    </row>
+    <row r="46" ht="22.5" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B46" s="3"/>
       <c r="D46" t="s">
-        <v>101</v>
+        <v>7</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="B47">
         <v>703</v>
@@ -1386,12 +1370,12 @@
         <v>1000</v>
       </c>
       <c r="D47" t="s">
-        <v>101</v>
+        <v>48</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="B48">
         <v>703</v>
@@ -1400,12 +1384,12 @@
         <v>1000</v>
       </c>
       <c r="D48" t="s">
-        <v>101</v>
+        <v>48</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="B49">
         <v>703</v>
@@ -1414,23 +1398,23 @@
         <v>1100</v>
       </c>
       <c r="D49" t="s">
-        <v>101</v>
+        <v>48</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C50">
         <v>900</v>
       </c>
       <c r="D50" t="s">
-        <v>101</v>
+        <v>48</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="B51">
         <v>900</v>
@@ -1439,136 +1423,136 @@
         <v>550</v>
       </c>
       <c r="D51" t="s">
-        <v>101</v>
+        <v>48</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="C52">
         <v>1200</v>
       </c>
       <c r="D52" t="s">
-        <v>101</v>
+        <v>48</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="C53">
         <v>1000</v>
       </c>
       <c r="D53" t="s">
-        <v>101</v>
+        <v>48</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="C54">
         <v>1000</v>
       </c>
       <c r="D54" t="s">
-        <v>101</v>
+        <v>48</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="C55">
         <v>1000</v>
       </c>
       <c r="D55" t="s">
-        <v>101</v>
+        <v>48</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="C56">
         <v>1600</v>
       </c>
       <c r="D56" t="s">
-        <v>101</v>
+        <v>48</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C57">
         <v>1100</v>
       </c>
       <c r="D57" t="s">
-        <v>101</v>
+        <v>48</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="C58">
         <v>1100</v>
       </c>
       <c r="D58" t="s">
-        <v>101</v>
+        <v>48</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="C59">
         <v>3000</v>
       </c>
       <c r="D59" t="s">
-        <v>101</v>
+        <v>48</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="C60">
         <v>2500</v>
       </c>
       <c r="D60" t="s">
-        <v>101</v>
+        <v>48</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="C61">
         <v>2000</v>
       </c>
       <c r="D61" t="s">
-        <v>101</v>
+        <v>48</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>7</v>
-      </c>
-      <c r="B62">
-        <v>1000</v>
+        <v>11</v>
+      </c>
+      <c r="B62" t="s">
+        <v>58</v>
       </c>
       <c r="C62">
         <v>1500</v>
       </c>
       <c r="D62" t="s">
-        <v>101</v>
+        <v>48</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="B63">
         <v>1000</v>
@@ -1577,12 +1561,12 @@
         <v>1500</v>
       </c>
       <c r="D63" t="s">
-        <v>101</v>
+        <v>48</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B64">
         <v>580</v>
@@ -1591,12 +1575,12 @@
         <v>1500</v>
       </c>
       <c r="D64" t="s">
-        <v>101</v>
+        <v>48</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="B65">
         <v>910</v>
@@ -1605,12 +1589,12 @@
         <v>1200</v>
       </c>
       <c r="D65" t="s">
-        <v>101</v>
+        <v>48</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="B66">
         <v>670</v>
@@ -1619,34 +1603,34 @@
         <v>1000</v>
       </c>
       <c r="D66" t="s">
-        <v>101</v>
+        <v>48</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C67">
         <v>1400</v>
       </c>
       <c r="D67" t="s">
-        <v>101</v>
+        <v>48</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="C68">
         <v>1000</v>
       </c>
       <c r="D68" t="s">
-        <v>101</v>
+        <v>48</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="B69">
         <v>900</v>
@@ -1655,161 +1639,161 @@
         <v>1200</v>
       </c>
       <c r="D69" t="s">
-        <v>101</v>
+        <v>48</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="C70">
         <v>3000</v>
       </c>
       <c r="D70" t="s">
-        <v>101</v>
+        <v>48</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="C71">
         <v>2500</v>
       </c>
       <c r="D71" t="s">
-        <v>101</v>
+        <v>48</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="C72">
         <v>950</v>
       </c>
       <c r="D72" t="s">
-        <v>101</v>
+        <v>48</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="C73">
         <v>1200</v>
       </c>
       <c r="D73" t="s">
-        <v>101</v>
+        <v>48</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="C74">
         <v>2200</v>
       </c>
       <c r="D74" t="s">
-        <v>101</v>
+        <v>48</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="C75">
         <v>1300</v>
       </c>
       <c r="D75" t="s">
-        <v>101</v>
+        <v>48</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="C76">
         <v>2600</v>
       </c>
       <c r="D76" t="s">
-        <v>101</v>
+        <v>48</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="C77">
         <v>2250</v>
       </c>
       <c r="D77" t="s">
-        <v>101</v>
+        <v>48</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="C78">
         <v>3500</v>
       </c>
       <c r="D78" t="s">
-        <v>101</v>
+        <v>48</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="C79">
         <v>4000</v>
       </c>
       <c r="D79" t="s">
-        <v>101</v>
+        <v>48</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="C80">
         <v>1000</v>
       </c>
       <c r="D80" t="s">
-        <v>101</v>
+        <v>48</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="C81">
         <v>1500</v>
       </c>
       <c r="D81" t="s">
-        <v>101</v>
+        <v>48</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="C82">
         <v>1800</v>
       </c>
       <c r="D82" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="83" spans="1:4" ht="22.5" x14ac:dyDescent="0.45">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="83" ht="22.5" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A83" s="5" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="B83" s="5"/>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="B84">
         <v>175</v>
@@ -1818,12 +1802,12 @@
         <v>250</v>
       </c>
       <c r="D84" t="s">
-        <v>102</v>
+        <v>72</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="B85">
         <v>175</v>
@@ -1832,12 +1816,12 @@
         <v>250</v>
       </c>
       <c r="D85" t="s">
-        <v>102</v>
+        <v>72</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="B86">
         <v>215</v>
@@ -1846,12 +1830,12 @@
         <v>300</v>
       </c>
       <c r="D86" t="s">
-        <v>102</v>
+        <v>72</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>66</v>
+        <v>75</v>
       </c>
       <c r="B87">
         <v>198</v>
@@ -1860,12 +1844,12 @@
         <v>300</v>
       </c>
       <c r="D87" t="s">
-        <v>102</v>
+        <v>72</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>67</v>
+        <v>76</v>
       </c>
       <c r="B88">
         <v>200</v>
@@ -1874,12 +1858,12 @@
         <v>300</v>
       </c>
       <c r="D88" t="s">
-        <v>102</v>
+        <v>72</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>68</v>
+        <v>77</v>
       </c>
       <c r="B89">
         <v>200</v>
@@ -1888,12 +1872,12 @@
         <v>300</v>
       </c>
       <c r="D89" t="s">
-        <v>102</v>
+        <v>72</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>69</v>
+        <v>78</v>
       </c>
       <c r="B90">
         <v>232</v>
@@ -1902,23 +1886,23 @@
         <v>300</v>
       </c>
       <c r="D90" t="s">
-        <v>102</v>
+        <v>72</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>70</v>
+        <v>79</v>
       </c>
       <c r="C91">
         <v>300</v>
       </c>
       <c r="D91" t="s">
-        <v>102</v>
+        <v>72</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>71</v>
+        <v>80</v>
       </c>
       <c r="B92">
         <v>175</v>
@@ -1927,56 +1911,56 @@
         <v>300</v>
       </c>
       <c r="D92" t="s">
-        <v>102</v>
+        <v>72</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
+        <v>81</v>
+      </c>
+      <c r="C93">
+        <v>300</v>
+      </c>
+      <c r="D93" t="s">
         <v>72</v>
-      </c>
-      <c r="C93">
-        <v>300</v>
-      </c>
-      <c r="D93" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="C94">
         <v>250</v>
       </c>
       <c r="D94" t="s">
-        <v>102</v>
+        <v>72</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="C95">
         <v>400</v>
       </c>
       <c r="D95" t="s">
-        <v>102</v>
+        <v>72</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>75</v>
+        <v>84</v>
       </c>
       <c r="C96">
         <v>300</v>
       </c>
       <c r="D96" t="s">
-        <v>102</v>
+        <v>72</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>106</v>
+        <v>85</v>
       </c>
       <c r="B97">
         <v>215</v>
@@ -1985,12 +1969,12 @@
         <v>300</v>
       </c>
       <c r="D97" t="s">
-        <v>102</v>
+        <v>72</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="B98">
         <v>600</v>
@@ -1999,12 +1983,12 @@
         <v>800</v>
       </c>
       <c r="D98" t="s">
-        <v>102</v>
+        <v>72</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="B99">
         <v>200</v>
@@ -2013,23 +1997,23 @@
         <v>270</v>
       </c>
       <c r="D99" t="s">
-        <v>102</v>
+        <v>72</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="C100">
         <v>400</v>
       </c>
       <c r="D100" t="s">
-        <v>102</v>
+        <v>72</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="B101">
         <v>198</v>
@@ -2038,23 +2022,23 @@
         <v>270</v>
       </c>
       <c r="D101" t="s">
-        <v>102</v>
+        <v>72</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="C102">
         <v>270</v>
       </c>
       <c r="D102" t="s">
-        <v>102</v>
+        <v>72</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>69</v>
+        <v>78</v>
       </c>
       <c r="B103">
         <v>234</v>
@@ -2063,166 +2047,166 @@
         <v>270</v>
       </c>
       <c r="D103" t="s">
-        <v>102</v>
+        <v>72</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="C104">
         <v>270</v>
       </c>
       <c r="D104" t="s">
-        <v>102</v>
+        <v>72</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>107</v>
+        <v>91</v>
       </c>
       <c r="C105">
         <v>270</v>
       </c>
       <c r="D105" t="s">
-        <v>103</v>
+        <v>92</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="C106">
         <v>300</v>
       </c>
       <c r="D106" t="s">
-        <v>103</v>
+        <v>92</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>82</v>
+        <v>94</v>
       </c>
       <c r="C107">
         <v>70</v>
       </c>
       <c r="D107" t="s">
-        <v>103</v>
+        <v>92</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>83</v>
+        <v>95</v>
       </c>
       <c r="C108">
         <v>50</v>
       </c>
       <c r="D108" t="s">
-        <v>103</v>
+        <v>92</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="C109">
         <v>40</v>
       </c>
       <c r="D109" t="s">
-        <v>103</v>
+        <v>92</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>85</v>
+        <v>97</v>
       </c>
       <c r="C110">
         <v>30</v>
       </c>
       <c r="D110" t="s">
-        <v>103</v>
+        <v>92</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="C111">
         <v>180</v>
       </c>
       <c r="D111" t="s">
-        <v>103</v>
+        <v>92</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="C112">
         <v>150</v>
       </c>
       <c r="D112" t="s">
-        <v>103</v>
+        <v>92</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>88</v>
+        <v>100</v>
       </c>
       <c r="C113">
         <v>200</v>
       </c>
       <c r="D113" t="s">
-        <v>103</v>
+        <v>92</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>89</v>
+        <v>101</v>
       </c>
       <c r="C114">
         <v>80</v>
       </c>
       <c r="D114" t="s">
-        <v>103</v>
+        <v>92</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>90</v>
+        <v>102</v>
       </c>
       <c r="C115">
         <v>160</v>
       </c>
       <c r="D115" t="s">
-        <v>103</v>
+        <v>92</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="C116">
         <v>70</v>
       </c>
       <c r="D116" t="s">
-        <v>103</v>
+        <v>92</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>92</v>
+        <v>104</v>
       </c>
       <c r="C117">
         <v>100</v>
       </c>
       <c r="D117" t="s">
-        <v>103</v>
+        <v>92</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="B118">
         <v>60</v>
@@ -2231,51 +2215,51 @@
         <v>50</v>
       </c>
       <c r="D118" t="s">
-        <v>103</v>
+        <v>92</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="C119">
         <v>70</v>
       </c>
       <c r="D119" t="s">
-        <v>103</v>
+        <v>92</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>95</v>
+        <v>107</v>
       </c>
       <c r="C120">
         <v>100</v>
       </c>
       <c r="D120" t="s">
-        <v>103</v>
+        <v>92</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>96</v>
+        <v>108</v>
       </c>
       <c r="C121">
         <v>30</v>
       </c>
       <c r="D121" t="s">
-        <v>103</v>
+        <v>92</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>97</v>
+        <v>109</v>
       </c>
       <c r="C122">
         <v>50</v>
       </c>
       <c r="D122" t="s">
-        <v>103</v>
+        <v>92</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add stock sheet and update price list data
</commit_message>
<xml_diff>
--- a/price list.xlsx
+++ b/price list.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="134">
   <si>
     <t>Product</t>
   </si>
@@ -37,138 +37,168 @@
     <t>Best Whiskey</t>
   </si>
   <si>
+    <t>250</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blue Ice </t>
+  </si>
+  <si>
+    <t>V&amp;A</t>
+  </si>
+  <si>
+    <t>Bond 7</t>
+  </si>
+  <si>
+    <t>320</t>
+  </si>
+  <si>
+    <t>viceroy</t>
+  </si>
+  <si>
+    <t>Smirnoff</t>
+  </si>
+  <si>
+    <t>350</t>
+  </si>
+  <si>
+    <t>Kane</t>
+  </si>
+  <si>
+    <t>Napoleon</t>
+  </si>
+  <si>
+    <t>185</t>
+  </si>
+  <si>
+    <t>Konyagi</t>
+  </si>
+  <si>
+    <t>Richot</t>
+  </si>
+  <si>
+    <t>358</t>
+  </si>
+  <si>
+    <t>Kenya King</t>
+  </si>
+  <si>
+    <t>Muckpit</t>
+  </si>
+  <si>
+    <t>Captain Morgan</t>
+  </si>
+  <si>
+    <t>Origin</t>
+  </si>
+  <si>
+    <t>Chrome Vodka</t>
+  </si>
+  <si>
+    <t>Tripple Ace</t>
+  </si>
+  <si>
+    <t>Kibao</t>
+  </si>
+  <si>
+    <t>Hunters</t>
+  </si>
+  <si>
+    <t>Best  Gin</t>
+  </si>
+  <si>
+    <t>William Grayson</t>
+  </si>
+  <si>
+    <t>Dallas</t>
+  </si>
+  <si>
+    <t>95</t>
+  </si>
+  <si>
+    <t>200</t>
+  </si>
+  <si>
+    <t>General Meakings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">People Vodka </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Smart Vodka </t>
+  </si>
+  <si>
+    <t>Best Vodka</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Chrome Gin</t>
+  </si>
+  <si>
+    <t>County</t>
+  </si>
+  <si>
+    <t>carribian</t>
+  </si>
+  <si>
+    <t>Trace</t>
+  </si>
+  <si>
+    <t>KC. Pineapple</t>
+  </si>
+  <si>
+    <t>Kc smooth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KC .Ginger </t>
+  </si>
+  <si>
+    <t>Brand 350ml</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
-    <t xml:space="preserve">Blue Ice </t>
-  </si>
-  <si>
-    <t>V&amp;A</t>
-  </si>
-  <si>
-    <t>Bond 7</t>
-  </si>
-  <si>
-    <t>viceroy</t>
-  </si>
-  <si>
-    <t>Smirnoff</t>
-  </si>
-  <si>
-    <t>Kane</t>
-  </si>
-  <si>
-    <t>Napoleon</t>
-  </si>
-  <si>
-    <t>Konyagi</t>
-  </si>
-  <si>
-    <t>Richot</t>
-  </si>
-  <si>
-    <t>Kenya King</t>
-  </si>
-  <si>
-    <t>Muckpit</t>
-  </si>
-  <si>
-    <t>Captain Morgan</t>
-  </si>
-  <si>
-    <t>Origin</t>
-  </si>
-  <si>
-    <t>Chrome Vodka</t>
-  </si>
-  <si>
-    <t>Tripple Ace</t>
-  </si>
-  <si>
-    <t>Kibao</t>
-  </si>
-  <si>
-    <t>Hunters</t>
-  </si>
-  <si>
-    <t>Best  Gin</t>
-  </si>
-  <si>
-    <t>William Grayson</t>
+    <t xml:space="preserve">Jameson </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>350ml</t>
+  </si>
+  <si>
+    <t>Black&amp;white</t>
+  </si>
+  <si>
+    <t>CrazyCork</t>
+  </si>
+  <si>
+    <t>650</t>
+  </si>
+  <si>
+    <t>Viceroy</t>
+  </si>
+  <si>
+    <t>375ml</t>
+  </si>
+  <si>
+    <t>VAT 69</t>
+  </si>
+  <si>
+    <t>750ml</t>
+  </si>
+  <si>
+    <t>Brand 750ml</t>
+  </si>
+  <si>
+    <t>Kc.Ginger</t>
+  </si>
+  <si>
+    <t>1300</t>
   </si>
   <si>
     <t xml:space="preserve">All seasons </t>
   </si>
   <si>
-    <t>General Meakings</t>
-  </si>
-  <si>
-    <t xml:space="preserve">People Vodka </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Smart Vodka </t>
-  </si>
-  <si>
-    <t>Best Vodka</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Chrome Gin</t>
-  </si>
-  <si>
-    <t>County</t>
-  </si>
-  <si>
-    <t>carribian</t>
-  </si>
-  <si>
-    <t>Trace</t>
-  </si>
-  <si>
-    <t>KC. Pineapple</t>
-  </si>
-  <si>
-    <t>Kc smooth</t>
-  </si>
-  <si>
-    <t xml:space="preserve">KC .Ginger </t>
-  </si>
-  <si>
-    <t>Brand 350ml</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jameson </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> </t>
-  </si>
-  <si>
-    <t>350ml</t>
-  </si>
-  <si>
-    <t>Black&amp;white</t>
-  </si>
-  <si>
-    <t>CrazyCork</t>
-  </si>
-  <si>
-    <t>Viceroy</t>
-  </si>
-  <si>
-    <t>375ml</t>
-  </si>
-  <si>
-    <t>VAT 69</t>
-  </si>
-  <si>
-    <t>750ml</t>
-  </si>
-  <si>
-    <t>Brand 750ml</t>
-  </si>
-  <si>
-    <t>Kc.Ginger</t>
-  </si>
-  <si>
     <t>Kenya king</t>
   </si>
   <si>
@@ -271,6 +301,15 @@
     <t>Balozi</t>
   </si>
   <si>
+    <t>245</t>
+  </si>
+  <si>
+    <t>Balozi Bottle</t>
+  </si>
+  <si>
+    <t>169</t>
+  </si>
+  <si>
     <t>Whitecup</t>
   </si>
   <si>
@@ -286,9 +325,30 @@
     <t>Tusker Bottle</t>
   </si>
   <si>
+    <t>Bottle</t>
+  </si>
+  <si>
+    <t>150</t>
+  </si>
+  <si>
+    <t>Guiness Bottle</t>
+  </si>
+  <si>
+    <t>204</t>
+  </si>
+  <si>
+    <t>270</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pilsner </t>
   </si>
   <si>
+    <t>195</t>
+  </si>
+  <si>
+    <t>pilsner bottle</t>
+  </si>
+  <si>
     <t>White Cup Bottle</t>
   </si>
   <si>
@@ -301,13 +361,25 @@
     <t>Soda 500ml</t>
   </si>
   <si>
+    <t>63</t>
+  </si>
+  <si>
     <t>Soda 350ml</t>
   </si>
   <si>
+    <t>41</t>
+  </si>
+  <si>
     <t>Soda 300ml</t>
   </si>
   <si>
+    <t>32</t>
+  </si>
+  <si>
     <t>Soda 200ml</t>
+  </si>
+  <si>
+    <t>25</t>
   </si>
   <si>
     <t>Soda 1.25ltrs</t>
@@ -753,7 +825,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D122"/>
+  <dimension ref="A1:D125"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="18" customWidth="1"/>
@@ -836,7 +908,7 @@
         <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="C6">
         <v>550</v>
@@ -847,7 +919,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B7">
         <v>395</v>
@@ -861,7 +933,10 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="B8" t="s">
+        <v>14</v>
       </c>
       <c r="C8">
         <v>500</v>
@@ -872,7 +947,7 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B9">
         <v>195</v>
@@ -886,7 +961,10 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>14</v>
+        <v>16</v>
+      </c>
+      <c r="B10" t="s">
+        <v>17</v>
       </c>
       <c r="C10">
         <v>300</v>
@@ -897,7 +975,7 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B11">
         <v>225</v>
@@ -911,7 +989,10 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>16</v>
+        <v>19</v>
+      </c>
+      <c r="B12" t="s">
+        <v>20</v>
       </c>
       <c r="C12">
         <v>550</v>
@@ -922,7 +1003,7 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B13">
         <v>95</v>
@@ -936,7 +1017,7 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="B14">
         <v>340</v>
@@ -950,7 +1031,7 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B15">
         <v>334</v>
@@ -964,7 +1045,7 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="B16">
         <v>232</v>
@@ -978,7 +1059,7 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B17">
         <v>208</v>
@@ -992,7 +1073,7 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="B18">
         <v>197</v>
@@ -1006,7 +1087,7 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="B19">
         <v>225</v>
@@ -1020,7 +1101,7 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="B20">
         <v>285</v>
@@ -1034,7 +1115,7 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B21" t="s">
         <v>7</v>
@@ -1048,7 +1129,7 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="B22">
         <v>200</v>
@@ -1062,10 +1143,13 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>27</v>
-      </c>
-      <c r="C23">
-        <v>600</v>
+        <v>31</v>
+      </c>
+      <c r="B23" t="s">
+        <v>32</v>
+      </c>
+      <c r="C23" t="s">
+        <v>33</v>
       </c>
       <c r="D23" t="s">
         <v>5</v>
@@ -1073,7 +1157,7 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="B24">
         <v>210</v>
@@ -1087,7 +1171,7 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="B25">
         <v>125</v>
@@ -1101,7 +1185,7 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="B26">
         <v>100</v>
@@ -1115,7 +1199,7 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="B27">
         <v>285</v>
@@ -1129,7 +1213,7 @@
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="B28">
         <v>210</v>
@@ -1143,7 +1227,7 @@
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="B29">
         <v>231</v>
@@ -1157,7 +1241,7 @@
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="B30">
         <v>200</v>
@@ -1171,7 +1255,7 @@
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="B31">
         <v>95</v>
@@ -1185,7 +1269,7 @@
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="B32">
         <v>256</v>
@@ -1199,7 +1283,7 @@
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="B33">
         <v>256</v>
@@ -1213,7 +1297,7 @@
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="B34">
         <v>256</v>
@@ -1227,44 +1311,44 @@
     </row>
     <row r="35" ht="18.75" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="4" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="B35" s="4"/>
       <c r="D35" t="s">
-        <v>7</v>
+        <v>46</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="C36" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="D36" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C37">
         <v>800</v>
       </c>
       <c r="D37" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="C38">
         <v>1100</v>
       </c>
       <c r="D38" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
@@ -1278,56 +1362,56 @@
         <v>850</v>
       </c>
       <c r="D39" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C40">
         <v>850</v>
       </c>
       <c r="D40" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="C41">
         <v>500</v>
       </c>
       <c r="D41" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="C42">
         <v>550</v>
       </c>
       <c r="D42" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>24</v>
-      </c>
-      <c r="C43">
-        <v>750</v>
+        <v>28</v>
+      </c>
+      <c r="C43" t="s">
+        <v>52</v>
       </c>
       <c r="D43" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="B44">
         <v>575</v>
@@ -1336,32 +1420,32 @@
         <v>800</v>
       </c>
       <c r="D44" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="C45">
         <v>800</v>
       </c>
       <c r="D45" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
     </row>
     <row r="46" ht="22.5" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="B46" s="3"/>
       <c r="D46" t="s">
-        <v>7</v>
+        <v>46</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="B47">
         <v>703</v>
@@ -1370,12 +1454,12 @@
         <v>1000</v>
       </c>
       <c r="D47" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="B48">
         <v>703</v>
@@ -1384,12 +1468,12 @@
         <v>1000</v>
       </c>
       <c r="D48" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="B49">
         <v>703</v>
@@ -1398,7 +1482,7 @@
         <v>1100</v>
       </c>
       <c r="D49" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
@@ -1409,150 +1493,150 @@
         <v>900</v>
       </c>
       <c r="D50" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="B51">
         <v>900</v>
       </c>
-      <c r="C51">
-        <v>550</v>
+      <c r="C51" t="s">
+        <v>59</v>
       </c>
       <c r="D51" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>27</v>
+        <v>60</v>
       </c>
       <c r="C52">
         <v>1200</v>
       </c>
       <c r="D52" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="C53">
         <v>1000</v>
       </c>
       <c r="D53" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C54">
         <v>1000</v>
       </c>
       <c r="D54" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="C55">
         <v>1000</v>
       </c>
       <c r="D55" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>53</v>
+        <v>63</v>
       </c>
       <c r="C56">
         <v>1600</v>
       </c>
       <c r="D56" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C57">
         <v>1100</v>
       </c>
       <c r="D57" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>54</v>
+        <v>64</v>
       </c>
       <c r="C58">
         <v>1100</v>
       </c>
       <c r="D58" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="C59">
         <v>3000</v>
       </c>
       <c r="D59" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>56</v>
+        <v>66</v>
       </c>
       <c r="C60">
         <v>2500</v>
       </c>
       <c r="D60" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>57</v>
+        <v>67</v>
       </c>
       <c r="C61">
         <v>2000</v>
       </c>
       <c r="D61" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B62" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="C62">
         <v>1500</v>
       </c>
       <c r="D62" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="B63">
         <v>1000</v>
@@ -1561,7 +1645,7 @@
         <v>1500</v>
       </c>
       <c r="D63" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
@@ -1575,12 +1659,12 @@
         <v>1500</v>
       </c>
       <c r="D64" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B65">
         <v>910</v>
@@ -1589,12 +1673,12 @@
         <v>1200</v>
       </c>
       <c r="D65" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="B66">
         <v>670</v>
@@ -1603,34 +1687,34 @@
         <v>1000</v>
       </c>
       <c r="D66" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C67">
         <v>1400</v>
       </c>
       <c r="D67" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="C68">
         <v>1000</v>
       </c>
       <c r="D68" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="B69">
         <v>900</v>
@@ -1639,161 +1723,161 @@
         <v>1200</v>
       </c>
       <c r="D69" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>59</v>
+        <v>69</v>
       </c>
       <c r="C70">
         <v>3000</v>
       </c>
       <c r="D70" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="C71">
         <v>2500</v>
       </c>
       <c r="D71" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>61</v>
+        <v>71</v>
       </c>
       <c r="C72">
         <v>950</v>
       </c>
       <c r="D72" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="C73">
         <v>1200</v>
       </c>
       <c r="D73" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="C74">
         <v>2200</v>
       </c>
       <c r="D74" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="C75">
         <v>1300</v>
       </c>
       <c r="D75" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="C76">
         <v>2600</v>
       </c>
       <c r="D76" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="C77">
         <v>2250</v>
       </c>
       <c r="D77" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="C78">
         <v>3500</v>
       </c>
       <c r="D78" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="C79">
         <v>4000</v>
       </c>
       <c r="D79" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="C80">
         <v>1000</v>
       </c>
       <c r="D80" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C81">
         <v>1500</v>
       </c>
       <c r="D81" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="C82">
         <v>1800</v>
       </c>
       <c r="D82" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
     </row>
     <row r="83" ht="22.5" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A83" s="5" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="B83" s="5"/>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="B84">
         <v>175</v>
@@ -1802,12 +1886,12 @@
         <v>250</v>
       </c>
       <c r="D84" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="B85">
         <v>175</v>
@@ -1816,12 +1900,12 @@
         <v>250</v>
       </c>
       <c r="D85" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="B86">
         <v>215</v>
@@ -1830,12 +1914,12 @@
         <v>300</v>
       </c>
       <c r="D86" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="B87">
         <v>198</v>
@@ -1844,12 +1928,12 @@
         <v>300</v>
       </c>
       <c r="D87" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="B88">
         <v>200</v>
@@ -1858,12 +1942,12 @@
         <v>300</v>
       </c>
       <c r="D88" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="B89">
         <v>200</v>
@@ -1872,12 +1956,12 @@
         <v>300</v>
       </c>
       <c r="D89" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="B90">
         <v>232</v>
@@ -1886,23 +1970,23 @@
         <v>300</v>
       </c>
       <c r="D90" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="C91">
         <v>300</v>
       </c>
       <c r="D91" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="B92">
         <v>175</v>
@@ -1911,355 +1995,415 @@
         <v>300</v>
       </c>
       <c r="D92" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="C93">
         <v>300</v>
       </c>
       <c r="D93" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="C94">
         <v>250</v>
       </c>
       <c r="D94" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>83</v>
+        <v>93</v>
       </c>
       <c r="C95">
         <v>400</v>
       </c>
       <c r="D95" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>84</v>
+        <v>94</v>
+      </c>
+      <c r="B96" t="s">
+        <v>95</v>
       </c>
       <c r="C96">
         <v>300</v>
       </c>
       <c r="D96" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>85</v>
-      </c>
-      <c r="B97">
-        <v>215</v>
-      </c>
-      <c r="C97">
-        <v>300</v>
+        <v>96</v>
+      </c>
+      <c r="B97" t="s">
+        <v>97</v>
+      </c>
+      <c r="C97" t="s">
+        <v>7</v>
       </c>
       <c r="D97" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="B98">
-        <v>600</v>
+        <v>215</v>
       </c>
       <c r="C98">
-        <v>800</v>
+        <v>300</v>
       </c>
       <c r="D98" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="B99">
-        <v>200</v>
+        <v>600</v>
       </c>
       <c r="C99">
-        <v>270</v>
+        <v>800</v>
       </c>
       <c r="D99" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>88</v>
+        <v>100</v>
+      </c>
+      <c r="B100">
+        <v>200</v>
       </c>
       <c r="C100">
-        <v>400</v>
+        <v>270</v>
       </c>
       <c r="D100" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>89</v>
-      </c>
-      <c r="B101">
-        <v>198</v>
+        <v>101</v>
+      </c>
+      <c r="B101" t="s">
+        <v>97</v>
       </c>
       <c r="C101">
-        <v>270</v>
+        <v>400</v>
       </c>
       <c r="D101" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>74</v>
+        <v>102</v>
+      </c>
+      <c r="B102">
+        <v>198</v>
       </c>
       <c r="C102">
         <v>270</v>
       </c>
       <c r="D102" t="s">
-        <v>72</v>
+        <v>103</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>78</v>
-      </c>
-      <c r="B103">
-        <v>234</v>
+        <v>84</v>
+      </c>
+      <c r="B103" t="s">
+        <v>104</v>
       </c>
       <c r="C103">
         <v>270</v>
       </c>
       <c r="D103" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>90</v>
-      </c>
-      <c r="C104">
-        <v>270</v>
+        <v>105</v>
+      </c>
+      <c r="B104" t="s">
+        <v>106</v>
+      </c>
+      <c r="C104" t="s">
+        <v>107</v>
       </c>
       <c r="D104" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>91</v>
+        <v>88</v>
+      </c>
+      <c r="B105">
+        <v>234</v>
       </c>
       <c r="C105">
         <v>270</v>
       </c>
       <c r="D105" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>93</v>
+        <v>108</v>
+      </c>
+      <c r="B106" t="s">
+        <v>109</v>
       </c>
       <c r="C106">
-        <v>300</v>
+        <v>270</v>
       </c>
       <c r="D106" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="107" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>94</v>
-      </c>
-      <c r="C107">
-        <v>70</v>
-      </c>
-      <c r="D107" t="s">
-        <v>92</v>
+        <v>110</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>95</v>
+        <v>111</v>
+      </c>
+      <c r="B108" t="s">
+        <v>109</v>
       </c>
       <c r="C108">
-        <v>50</v>
+        <v>270</v>
       </c>
       <c r="D108" t="s">
-        <v>92</v>
+        <v>112</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>96</v>
+        <v>113</v>
       </c>
       <c r="C109">
-        <v>40</v>
+        <v>300</v>
       </c>
       <c r="D109" t="s">
-        <v>92</v>
+        <v>112</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>97</v>
+        <v>114</v>
+      </c>
+      <c r="B110" t="s">
+        <v>115</v>
       </c>
       <c r="C110">
-        <v>30</v>
+        <v>70</v>
       </c>
       <c r="D110" t="s">
-        <v>92</v>
+        <v>112</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>98</v>
+        <v>116</v>
+      </c>
+      <c r="B111" t="s">
+        <v>117</v>
       </c>
       <c r="C111">
-        <v>180</v>
+        <v>50</v>
       </c>
       <c r="D111" t="s">
-        <v>92</v>
+        <v>112</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>99</v>
+        <v>118</v>
+      </c>
+      <c r="B112" t="s">
+        <v>119</v>
       </c>
       <c r="C112">
-        <v>150</v>
+        <v>40</v>
       </c>
       <c r="D112" t="s">
-        <v>92</v>
+        <v>112</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>100</v>
+        <v>120</v>
+      </c>
+      <c r="B113" t="s">
+        <v>121</v>
       </c>
       <c r="C113">
-        <v>200</v>
+        <v>30</v>
       </c>
       <c r="D113" t="s">
-        <v>92</v>
+        <v>112</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>101</v>
+        <v>122</v>
       </c>
       <c r="C114">
-        <v>80</v>
+        <v>180</v>
       </c>
       <c r="D114" t="s">
-        <v>92</v>
+        <v>112</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>102</v>
+        <v>123</v>
       </c>
       <c r="C115">
-        <v>160</v>
+        <v>150</v>
       </c>
       <c r="D115" t="s">
-        <v>92</v>
+        <v>112</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>103</v>
+        <v>124</v>
       </c>
       <c r="C116">
-        <v>70</v>
+        <v>200</v>
       </c>
       <c r="D116" t="s">
-        <v>92</v>
+        <v>112</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>104</v>
+        <v>125</v>
       </c>
       <c r="C117">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="D117" t="s">
-        <v>92</v>
+        <v>112</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>105</v>
-      </c>
-      <c r="B118">
-        <v>60</v>
+        <v>126</v>
       </c>
       <c r="C118">
-        <v>50</v>
+        <v>160</v>
       </c>
       <c r="D118" t="s">
-        <v>92</v>
+        <v>112</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>106</v>
+        <v>127</v>
       </c>
       <c r="C119">
         <v>70</v>
       </c>
       <c r="D119" t="s">
-        <v>92</v>
+        <v>112</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>107</v>
+        <v>128</v>
       </c>
       <c r="C120">
         <v>100</v>
       </c>
       <c r="D120" t="s">
-        <v>92</v>
+        <v>112</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>108</v>
+        <v>129</v>
+      </c>
+      <c r="B121">
+        <v>60</v>
       </c>
       <c r="C121">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="D121" t="s">
-        <v>92</v>
+        <v>112</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>109</v>
+        <v>130</v>
       </c>
       <c r="C122">
+        <v>70</v>
+      </c>
+      <c r="D122" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>131</v>
+      </c>
+      <c r="C123">
+        <v>100</v>
+      </c>
+      <c r="D123" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>132</v>
+      </c>
+      <c r="C124">
+        <v>30</v>
+      </c>
+      <c r="D124" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>133</v>
+      </c>
+      <c r="C125">
         <v>50</v>
       </c>
-      <c r="D122" t="s">
-        <v>92</v>
+      <c r="D125" t="s">
+        <v>112</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add daily expenses (net profit) and category picker for custom items
- New DailyExpense model; daily sales form now collects expenses and net profit = sales profit - expenses, reflected in report and Excel exports
- Custom items get a category dropdown and saved products persist in the sales list
- Update price list data
</commit_message>
<xml_diff>
--- a/price list.xlsx
+++ b/price list.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="141">
   <si>
     <t>Product</t>
   </si>
@@ -43,6 +43,9 @@
     <t xml:space="preserve">Blue Ice </t>
   </si>
   <si>
+    <t>95</t>
+  </si>
+  <si>
     <t>V&amp;A</t>
   </si>
   <si>
@@ -112,9 +115,6 @@
     <t>Dallas</t>
   </si>
   <si>
-    <t>95</t>
-  </si>
-  <si>
     <t>200</t>
   </si>
   <si>
@@ -193,6 +193,9 @@
     <t>Kc.Ginger</t>
   </si>
   <si>
+    <t>1000</t>
+  </si>
+  <si>
     <t>1300</t>
   </si>
   <si>
@@ -223,6 +226,12 @@
     <t>1200</t>
   </si>
   <si>
+    <t>600</t>
+  </si>
+  <si>
+    <t>900</t>
+  </si>
+  <si>
     <t>Amarula 1ltr</t>
   </si>
   <si>
@@ -400,19 +409,31 @@
     <t>Dasani Small</t>
   </si>
   <si>
+    <t>40</t>
+  </si>
+  <si>
     <t>Dasani Big</t>
   </si>
   <si>
+    <t>50</t>
+  </si>
+  <si>
     <t>Lemonade</t>
   </si>
   <si>
     <t>predator</t>
   </si>
   <si>
+    <t>46</t>
+  </si>
+  <si>
     <t>Kiss</t>
   </si>
   <si>
     <t>Glacier Small</t>
+  </si>
+  <si>
+    <t>20</t>
   </si>
   <si>
     <t>Glacier Big</t>
@@ -879,8 +900,8 @@
       <c r="A4" t="s">
         <v>8</v>
       </c>
-      <c r="B4">
-        <v>150</v>
+      <c r="B4" t="s">
+        <v>9</v>
       </c>
       <c r="C4">
         <v>160</v>
@@ -891,7 +912,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B5">
         <v>295</v>
@@ -905,10 +926,10 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C6">
         <v>550</v>
@@ -919,7 +940,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B7">
         <v>395</v>
@@ -933,10 +954,10 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B8" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C8">
         <v>500</v>
@@ -947,7 +968,7 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B9">
         <v>195</v>
@@ -961,10 +982,10 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B10" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C10">
         <v>300</v>
@@ -975,7 +996,7 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B11">
         <v>225</v>
@@ -989,10 +1010,10 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B12" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C12">
         <v>550</v>
@@ -1003,7 +1024,7 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B13">
         <v>95</v>
@@ -1017,7 +1038,7 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B14">
         <v>340</v>
@@ -1031,7 +1052,7 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B15">
         <v>334</v>
@@ -1045,7 +1066,7 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B16">
         <v>232</v>
@@ -1059,7 +1080,7 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B17">
         <v>208</v>
@@ -1073,7 +1094,7 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B18">
         <v>197</v>
@@ -1087,7 +1108,7 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B19">
         <v>225</v>
@@ -1101,7 +1122,7 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B20">
         <v>285</v>
@@ -1115,7 +1136,7 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B21" t="s">
         <v>7</v>
@@ -1129,7 +1150,7 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B22">
         <v>200</v>
@@ -1143,10 +1164,10 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B23" t="s">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="C23" t="s">
         <v>33</v>
@@ -1331,7 +1352,7 @@
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C37">
         <v>800</v>
@@ -1367,7 +1388,7 @@
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C40">
         <v>850</v>
@@ -1378,7 +1399,7 @@
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C41">
         <v>500</v>
@@ -1400,7 +1421,7 @@
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C43" t="s">
         <v>52</v>
@@ -1478,8 +1499,8 @@
       <c r="B49">
         <v>703</v>
       </c>
-      <c r="C49">
-        <v>1100</v>
+      <c r="C49" t="s">
+        <v>59</v>
       </c>
       <c r="D49" t="s">
         <v>56</v>
@@ -1487,7 +1508,7 @@
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C50">
         <v>900</v>
@@ -1498,13 +1519,13 @@
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B51">
         <v>900</v>
       </c>
       <c r="C51" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D51" t="s">
         <v>56</v>
@@ -1512,7 +1533,7 @@
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C52">
         <v>1200</v>
@@ -1523,7 +1544,7 @@
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C53">
         <v>1000</v>
@@ -1534,7 +1555,7 @@
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C54">
         <v>1000</v>
@@ -1545,7 +1566,7 @@
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C55">
         <v>1000</v>
@@ -1556,7 +1577,7 @@
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C56">
         <v>1600</v>
@@ -1567,7 +1588,7 @@
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C57">
         <v>1100</v>
@@ -1578,7 +1599,7 @@
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C58">
         <v>1100</v>
@@ -1589,7 +1610,7 @@
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C59">
         <v>3000</v>
@@ -1600,7 +1621,7 @@
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C60">
         <v>2500</v>
@@ -1611,7 +1632,7 @@
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C61">
         <v>2000</v>
@@ -1622,10 +1643,10 @@
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B62" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C62">
         <v>1500</v>
@@ -1664,7 +1685,7 @@
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B65">
         <v>910</v>
@@ -1692,7 +1713,7 @@
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C67">
         <v>1400</v>
@@ -1703,7 +1724,7 @@
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C68">
         <v>1000</v>
@@ -1716,11 +1737,11 @@
       <c r="A69" t="s">
         <v>34</v>
       </c>
-      <c r="B69">
-        <v>900</v>
-      </c>
-      <c r="C69">
-        <v>1200</v>
+      <c r="B69" t="s">
+        <v>70</v>
+      </c>
+      <c r="C69" t="s">
+        <v>71</v>
       </c>
       <c r="D69" t="s">
         <v>56</v>
@@ -1728,7 +1749,7 @@
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C70">
         <v>3000</v>
@@ -1739,7 +1760,7 @@
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="C71">
         <v>2500</v>
@@ -1750,7 +1771,7 @@
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="C72">
         <v>950</v>
@@ -1761,7 +1782,7 @@
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C73">
         <v>1200</v>
@@ -1772,7 +1793,7 @@
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C74">
         <v>2200</v>
@@ -1783,7 +1804,7 @@
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C75">
         <v>1300</v>
@@ -1794,7 +1815,7 @@
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="C76">
         <v>2600</v>
@@ -1805,7 +1826,7 @@
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="C77">
         <v>2250</v>
@@ -1816,7 +1837,7 @@
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="C78">
         <v>3500</v>
@@ -1827,7 +1848,7 @@
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="C79">
         <v>4000</v>
@@ -1838,7 +1859,7 @@
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="C80">
         <v>1000</v>
@@ -1849,7 +1870,7 @@
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C81">
         <v>1500</v>
@@ -1871,13 +1892,13 @@
     </row>
     <row r="83" ht="22.5" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A83" s="5" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B83" s="5"/>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B84">
         <v>175</v>
@@ -1886,12 +1907,12 @@
         <v>250</v>
       </c>
       <c r="D84" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B85">
         <v>175</v>
@@ -1900,12 +1921,12 @@
         <v>250</v>
       </c>
       <c r="D85" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="B86">
         <v>215</v>
@@ -1914,12 +1935,12 @@
         <v>300</v>
       </c>
       <c r="D86" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B87">
         <v>198</v>
@@ -1928,12 +1949,12 @@
         <v>300</v>
       </c>
       <c r="D87" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="B88">
         <v>200</v>
@@ -1942,12 +1963,12 @@
         <v>300</v>
       </c>
       <c r="D88" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B89">
         <v>200</v>
@@ -1956,12 +1977,12 @@
         <v>300</v>
       </c>
       <c r="D89" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="B90">
         <v>232</v>
@@ -1970,23 +1991,23 @@
         <v>300</v>
       </c>
       <c r="D90" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="C91">
         <v>300</v>
       </c>
       <c r="D91" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="B92">
         <v>175</v>
@@ -1995,73 +2016,73 @@
         <v>300</v>
       </c>
       <c r="D92" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="C93">
         <v>300</v>
       </c>
       <c r="D93" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="C94">
         <v>250</v>
       </c>
       <c r="D94" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="C95">
         <v>400</v>
       </c>
       <c r="D95" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="B96" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="C96">
         <v>300</v>
       </c>
       <c r="D96" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="B97" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="C97" t="s">
         <v>7</v>
       </c>
       <c r="D97" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="B98">
         <v>215</v>
@@ -2070,12 +2091,12 @@
         <v>300</v>
       </c>
       <c r="D98" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B99">
         <v>600</v>
@@ -2084,12 +2105,12 @@
         <v>800</v>
       </c>
       <c r="D99" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="B100">
         <v>200</v>
@@ -2098,26 +2119,26 @@
         <v>270</v>
       </c>
       <c r="D100" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="B101" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="C101">
         <v>400</v>
       </c>
       <c r="D101" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="B102">
         <v>198</v>
@@ -2126,40 +2147,40 @@
         <v>270</v>
       </c>
       <c r="D102" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="B103" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="C103">
         <v>270</v>
       </c>
       <c r="D103" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="B104" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="C104" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="D104" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="B105">
         <v>234</v>
@@ -2168,189 +2189,195 @@
         <v>270</v>
       </c>
       <c r="D105" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="B106" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="C106">
         <v>270</v>
       </c>
       <c r="D106" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="107" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="B108" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="C108">
         <v>270</v>
       </c>
       <c r="D108" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="C109">
         <v>300</v>
       </c>
       <c r="D109" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="B110" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="C110">
         <v>70</v>
       </c>
       <c r="D110" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="B111" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="C111">
         <v>50</v>
       </c>
       <c r="D111" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="B112" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="C112">
         <v>40</v>
       </c>
       <c r="D112" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="B113" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="C113">
         <v>30</v>
       </c>
       <c r="D113" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="C114">
         <v>180</v>
       </c>
       <c r="D114" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="C115">
         <v>150</v>
       </c>
       <c r="D115" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="C116">
         <v>200</v>
       </c>
       <c r="D116" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="C117">
         <v>80</v>
       </c>
       <c r="D117" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="C118">
         <v>160</v>
       </c>
       <c r="D118" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>127</v>
+        <v>130</v>
+      </c>
+      <c r="B119" t="s">
+        <v>131</v>
       </c>
       <c r="C119">
         <v>70</v>
       </c>
       <c r="D119" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>128</v>
+        <v>132</v>
+      </c>
+      <c r="B120" t="s">
+        <v>133</v>
       </c>
       <c r="C120">
         <v>100</v>
       </c>
       <c r="D120" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="B121">
         <v>60</v>
@@ -2359,51 +2386,60 @@
         <v>50</v>
       </c>
       <c r="D121" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>130</v>
+        <v>135</v>
+      </c>
+      <c r="B122" t="s">
+        <v>136</v>
       </c>
       <c r="C122">
         <v>70</v>
       </c>
       <c r="D122" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="C123">
         <v>100</v>
       </c>
       <c r="D123" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>132</v>
+        <v>138</v>
+      </c>
+      <c r="B124" t="s">
+        <v>139</v>
       </c>
       <c r="C124">
         <v>30</v>
       </c>
       <c r="D124" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
-        <v>133</v>
+        <v>140</v>
+      </c>
+      <c r="B125" t="s">
+        <v>124</v>
       </c>
       <c r="C125">
         <v>50</v>
       </c>
       <c r="D125" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sync daily sales (stck) sheet to updated price list
</commit_message>
<xml_diff>
--- a/price list.xlsx
+++ b/price list.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="132">
   <si>
     <t>Product</t>
   </si>
@@ -34,289 +34,262 @@
     <t>250ml</t>
   </si>
   <si>
-    <t>Best Whiskey</t>
+    <t xml:space="preserve">Blue Ice </t>
+  </si>
+  <si>
+    <t>95</t>
+  </si>
+  <si>
+    <t>V&amp;A</t>
+  </si>
+  <si>
+    <t>viceroy</t>
+  </si>
+  <si>
+    <t>Smirnoff</t>
+  </si>
+  <si>
+    <t>350</t>
+  </si>
+  <si>
+    <t>Kane</t>
+  </si>
+  <si>
+    <t>Napoleon</t>
+  </si>
+  <si>
+    <t>185</t>
+  </si>
+  <si>
+    <t>Konyagi</t>
+  </si>
+  <si>
+    <t>Richot</t>
+  </si>
+  <si>
+    <t>358</t>
+  </si>
+  <si>
+    <t>Captain Morgan</t>
+  </si>
+  <si>
+    <t>Origin</t>
+  </si>
+  <si>
+    <t>Chrome Vodka</t>
+  </si>
+  <si>
+    <t>Tripple Ace</t>
+  </si>
+  <si>
+    <t>Kibao</t>
+  </si>
+  <si>
+    <t>Hunters</t>
+  </si>
+  <si>
+    <t>William Grayson</t>
+  </si>
+  <si>
+    <t>Dallas</t>
+  </si>
+  <si>
+    <t>200</t>
+  </si>
+  <si>
+    <t>General Meakings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">People Vodka </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Smart Vodka </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Chrome Gin</t>
+  </si>
+  <si>
+    <t>County</t>
+  </si>
+  <si>
+    <t>Trace</t>
+  </si>
+  <si>
+    <t>KC. Pineapple</t>
+  </si>
+  <si>
+    <t>Kc smooth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KC .Ginger </t>
+  </si>
+  <si>
+    <t>Brand 350ml</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t xml:space="preserve">Jameson </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>350ml</t>
+  </si>
+  <si>
+    <t>Black&amp;white</t>
+  </si>
+  <si>
+    <t>650</t>
+  </si>
+  <si>
+    <t>Viceroy</t>
+  </si>
+  <si>
+    <t>375ml</t>
+  </si>
+  <si>
+    <t>VAT 69</t>
+  </si>
+  <si>
+    <t>750ml</t>
+  </si>
+  <si>
+    <t>Brand 750ml</t>
+  </si>
+  <si>
+    <t>Kc.Ginger</t>
+  </si>
+  <si>
+    <t>1000</t>
+  </si>
+  <si>
+    <t>1300</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All seasons </t>
+  </si>
+  <si>
+    <t>Kenya king</t>
+  </si>
+  <si>
+    <t>Chrome Gin</t>
+  </si>
+  <si>
+    <t>Imperial Blue</t>
+  </si>
+  <si>
+    <t>4th street</t>
+  </si>
+  <si>
+    <t>jameson 1l</t>
+  </si>
+  <si>
+    <t>Jameson 750ml</t>
+  </si>
+  <si>
+    <t>William Lawsons</t>
+  </si>
+  <si>
+    <t>1200</t>
+  </si>
+  <si>
+    <t>600</t>
+  </si>
+  <si>
+    <t>900</t>
+  </si>
+  <si>
+    <t>Amarula 1ltr</t>
+  </si>
+  <si>
+    <t>Amarula 750</t>
+  </si>
+  <si>
+    <t>Best Gin</t>
+  </si>
+  <si>
+    <t>Best Whisky</t>
+  </si>
+  <si>
+    <t>Red label 750</t>
+  </si>
+  <si>
+    <t>Red label 375ml</t>
+  </si>
+  <si>
+    <t>Red Label 1 ltr</t>
+  </si>
+  <si>
+    <t>Black Label 375ml</t>
+  </si>
+  <si>
+    <t>Black Label 750ml</t>
+  </si>
+  <si>
+    <t>Black Label 1ltr</t>
+  </si>
+  <si>
+    <t>Drostody hol</t>
+  </si>
+  <si>
+    <t>Cans</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Guarana </t>
+  </si>
+  <si>
+    <t>cans</t>
+  </si>
+  <si>
+    <t>Guarana Black</t>
+  </si>
+  <si>
+    <t>Guiness</t>
+  </si>
+  <si>
+    <t>Tusker</t>
+  </si>
+  <si>
+    <t>Tusker Malt</t>
+  </si>
+  <si>
+    <t>Tusker Lite</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tusker cider </t>
+  </si>
+  <si>
+    <t>Snapp</t>
+  </si>
+  <si>
+    <t>pineapple Punch</t>
+  </si>
+  <si>
+    <t>Faxe</t>
+  </si>
+  <si>
+    <t>Redbull</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Delmonte </t>
+  </si>
+  <si>
+    <t>Balozi</t>
+  </si>
+  <si>
+    <t>245</t>
+  </si>
+  <si>
+    <t>Balozi Bottle</t>
+  </si>
+  <si>
+    <t>169</t>
   </si>
   <si>
     <t>250</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Blue Ice </t>
-  </si>
-  <si>
-    <t>95</t>
-  </si>
-  <si>
-    <t>V&amp;A</t>
-  </si>
-  <si>
-    <t>Bond 7</t>
-  </si>
-  <si>
-    <t>320</t>
-  </si>
-  <si>
-    <t>viceroy</t>
-  </si>
-  <si>
-    <t>Smirnoff</t>
-  </si>
-  <si>
-    <t>350</t>
-  </si>
-  <si>
-    <t>Kane</t>
-  </si>
-  <si>
-    <t>Napoleon</t>
-  </si>
-  <si>
-    <t>185</t>
-  </si>
-  <si>
-    <t>Konyagi</t>
-  </si>
-  <si>
-    <t>Richot</t>
-  </si>
-  <si>
-    <t>358</t>
-  </si>
-  <si>
-    <t>Kenya King</t>
-  </si>
-  <si>
-    <t>Muckpit</t>
-  </si>
-  <si>
-    <t>Captain Morgan</t>
-  </si>
-  <si>
-    <t>Origin</t>
-  </si>
-  <si>
-    <t>Chrome Vodka</t>
-  </si>
-  <si>
-    <t>Tripple Ace</t>
-  </si>
-  <si>
-    <t>Kibao</t>
-  </si>
-  <si>
-    <t>Hunters</t>
-  </si>
-  <si>
-    <t>Best  Gin</t>
-  </si>
-  <si>
-    <t>William Grayson</t>
-  </si>
-  <si>
-    <t>Dallas</t>
-  </si>
-  <si>
-    <t>200</t>
-  </si>
-  <si>
-    <t>General Meakings</t>
-  </si>
-  <si>
-    <t xml:space="preserve">People Vodka </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Smart Vodka </t>
-  </si>
-  <si>
-    <t>Best Vodka</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Chrome Gin</t>
-  </si>
-  <si>
-    <t>County</t>
-  </si>
-  <si>
-    <t>carribian</t>
-  </si>
-  <si>
-    <t>Trace</t>
-  </si>
-  <si>
-    <t>KC. Pineapple</t>
-  </si>
-  <si>
-    <t>Kc smooth</t>
-  </si>
-  <si>
-    <t xml:space="preserve">KC .Ginger </t>
-  </si>
-  <si>
-    <t>Brand 350ml</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t xml:space="preserve">Jameson </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> </t>
-  </si>
-  <si>
-    <t>350ml</t>
-  </si>
-  <si>
-    <t>Black&amp;white</t>
-  </si>
-  <si>
-    <t>CrazyCork</t>
-  </si>
-  <si>
-    <t>650</t>
-  </si>
-  <si>
-    <t>Viceroy</t>
-  </si>
-  <si>
-    <t>375ml</t>
-  </si>
-  <si>
-    <t>VAT 69</t>
-  </si>
-  <si>
-    <t>750ml</t>
-  </si>
-  <si>
-    <t>Brand 750ml</t>
-  </si>
-  <si>
-    <t>Kc.Ginger</t>
-  </si>
-  <si>
-    <t>1000</t>
-  </si>
-  <si>
-    <t>1300</t>
-  </si>
-  <si>
-    <t xml:space="preserve">All seasons </t>
-  </si>
-  <si>
-    <t>Kenya king</t>
-  </si>
-  <si>
-    <t>Chrome Gin</t>
-  </si>
-  <si>
-    <t>Imperial Blue</t>
-  </si>
-  <si>
-    <t>4th street</t>
-  </si>
-  <si>
-    <t>jameson 1l</t>
-  </si>
-  <si>
-    <t>Jameson 750ml</t>
-  </si>
-  <si>
-    <t>William Lawsons</t>
-  </si>
-  <si>
-    <t>1200</t>
-  </si>
-  <si>
-    <t>600</t>
-  </si>
-  <si>
-    <t>900</t>
-  </si>
-  <si>
-    <t>Amarula 1ltr</t>
-  </si>
-  <si>
-    <t>Amarula 750</t>
-  </si>
-  <si>
-    <t>Best Gin</t>
-  </si>
-  <si>
-    <t>Best Whisky</t>
-  </si>
-  <si>
-    <t>Red label 750</t>
-  </si>
-  <si>
-    <t>Red label 375ml</t>
-  </si>
-  <si>
-    <t>Red Label 1 ltr</t>
-  </si>
-  <si>
-    <t>Black Label 375ml</t>
-  </si>
-  <si>
-    <t>Black Label 750ml</t>
-  </si>
-  <si>
-    <t>Black Label 1ltr</t>
-  </si>
-  <si>
-    <t>Drostody hol</t>
-  </si>
-  <si>
-    <t>Cans</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Guarana </t>
-  </si>
-  <si>
-    <t>cans</t>
-  </si>
-  <si>
-    <t>Guarana Black</t>
-  </si>
-  <si>
-    <t>Guiness</t>
-  </si>
-  <si>
-    <t>Tusker</t>
-  </si>
-  <si>
-    <t>Tusker Malt</t>
-  </si>
-  <si>
-    <t>Tusker Lite</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tusker cider </t>
-  </si>
-  <si>
-    <t>Snapp</t>
-  </si>
-  <si>
-    <t>pineapple Punch</t>
-  </si>
-  <si>
-    <t>Faxe</t>
-  </si>
-  <si>
-    <t>Redbull</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Delmonte </t>
-  </si>
-  <si>
-    <t>Balozi</t>
-  </si>
-  <si>
-    <t>245</t>
-  </si>
-  <si>
-    <t>Balozi Bottle</t>
-  </si>
-  <si>
-    <t>169</t>
   </si>
   <si>
     <t>Whitecup</t>
@@ -846,7 +819,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D125"/>
+  <dimension ref="A1:D117"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="18" customWidth="1"/>
@@ -890,7 +863,7 @@
         <v>7</v>
       </c>
       <c r="C3">
-        <v>450</v>
+        <v>160</v>
       </c>
       <c r="D3" t="s">
         <v>5</v>
@@ -900,11 +873,11 @@
       <c r="A4" t="s">
         <v>8</v>
       </c>
-      <c r="B4" t="s">
-        <v>9</v>
+      <c r="B4">
+        <v>295</v>
       </c>
       <c r="C4">
-        <v>160</v>
+        <v>300</v>
       </c>
       <c r="D4" t="s">
         <v>5</v>
@@ -912,13 +885,13 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B5">
-        <v>295</v>
+        <v>395</v>
       </c>
       <c r="C5">
-        <v>300</v>
+        <v>550</v>
       </c>
       <c r="D5" t="s">
         <v>5</v>
@@ -926,13 +899,13 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" t="s">
         <v>11</v>
       </c>
-      <c r="B6" t="s">
-        <v>12</v>
-      </c>
       <c r="C6">
-        <v>550</v>
+        <v>500</v>
       </c>
       <c r="D6" t="s">
         <v>5</v>
@@ -940,13 +913,13 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B7">
-        <v>395</v>
+        <v>195</v>
       </c>
       <c r="C7">
-        <v>550</v>
+        <v>300</v>
       </c>
       <c r="D7" t="s">
         <v>5</v>
@@ -954,13 +927,13 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" t="s">
         <v>14</v>
       </c>
-      <c r="B8" t="s">
-        <v>15</v>
-      </c>
       <c r="C8">
-        <v>500</v>
+        <v>300</v>
       </c>
       <c r="D8" t="s">
         <v>5</v>
@@ -968,10 +941,10 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B9">
-        <v>195</v>
+        <v>225</v>
       </c>
       <c r="C9">
         <v>300</v>
@@ -982,13 +955,13 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" t="s">
         <v>17</v>
       </c>
-      <c r="B10" t="s">
-        <v>18</v>
-      </c>
       <c r="C10">
-        <v>300</v>
+        <v>550</v>
       </c>
       <c r="D10" t="s">
         <v>5</v>
@@ -996,13 +969,13 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B11">
-        <v>225</v>
+        <v>334</v>
       </c>
       <c r="C11">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="D11" t="s">
         <v>5</v>
@@ -1010,13 +983,13 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>20</v>
-      </c>
-      <c r="B12" t="s">
-        <v>21</v>
+        <v>19</v>
+      </c>
+      <c r="B12">
+        <v>232</v>
       </c>
       <c r="C12">
-        <v>550</v>
+        <v>300</v>
       </c>
       <c r="D12" t="s">
         <v>5</v>
@@ -1024,13 +997,13 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B13">
-        <v>95</v>
+        <v>208</v>
       </c>
       <c r="C13">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="D13" t="s">
         <v>5</v>
@@ -1038,13 +1011,13 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B14">
-        <v>340</v>
+        <v>197</v>
       </c>
       <c r="C14">
-        <v>450</v>
+        <v>300</v>
       </c>
       <c r="D14" t="s">
         <v>5</v>
@@ -1052,13 +1025,13 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B15">
-        <v>334</v>
+        <v>225</v>
       </c>
       <c r="C15">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="D15" t="s">
         <v>5</v>
@@ -1066,13 +1039,13 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B16">
-        <v>232</v>
+        <v>285</v>
       </c>
       <c r="C16">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="D16" t="s">
         <v>5</v>
@@ -1080,10 +1053,10 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B17">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C17">
         <v>300</v>
@@ -1094,13 +1067,13 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>27</v>
-      </c>
-      <c r="B18">
-        <v>197</v>
-      </c>
-      <c r="C18">
-        <v>300</v>
+        <v>25</v>
+      </c>
+      <c r="B18" t="s">
+        <v>7</v>
+      </c>
+      <c r="C18" t="s">
+        <v>26</v>
       </c>
       <c r="D18" t="s">
         <v>5</v>
@@ -1108,10 +1081,10 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B19">
-        <v>225</v>
+        <v>210</v>
       </c>
       <c r="C19">
         <v>300</v>
@@ -1122,13 +1095,13 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B20">
-        <v>285</v>
+        <v>125</v>
       </c>
       <c r="C20">
-        <v>400</v>
+        <v>160</v>
       </c>
       <c r="D20" t="s">
         <v>5</v>
@@ -1136,13 +1109,13 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>30</v>
-      </c>
-      <c r="B21" t="s">
-        <v>7</v>
+        <v>29</v>
+      </c>
+      <c r="B21">
+        <v>100</v>
       </c>
       <c r="C21">
-        <v>400</v>
+        <v>160</v>
       </c>
       <c r="D21" t="s">
         <v>5</v>
@@ -1150,10 +1123,10 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B22">
-        <v>200</v>
+        <v>210</v>
       </c>
       <c r="C22">
         <v>300</v>
@@ -1164,13 +1137,13 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>32</v>
-      </c>
-      <c r="B23" t="s">
-        <v>9</v>
-      </c>
-      <c r="C23" t="s">
-        <v>33</v>
+        <v>31</v>
+      </c>
+      <c r="B23">
+        <v>231</v>
+      </c>
+      <c r="C23">
+        <v>300</v>
       </c>
       <c r="D23" t="s">
         <v>5</v>
@@ -1178,13 +1151,13 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B24">
-        <v>210</v>
+        <v>95</v>
       </c>
       <c r="C24">
-        <v>300</v>
+        <v>160</v>
       </c>
       <c r="D24" t="s">
         <v>5</v>
@@ -1192,13 +1165,13 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B25">
-        <v>125</v>
+        <v>256</v>
       </c>
       <c r="C25">
-        <v>160</v>
+        <v>330</v>
       </c>
       <c r="D25" t="s">
         <v>5</v>
@@ -1206,13 +1179,13 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B26">
-        <v>100</v>
+        <v>256</v>
       </c>
       <c r="C26">
-        <v>160</v>
+        <v>330</v>
       </c>
       <c r="D26" t="s">
         <v>5</v>
@@ -1220,931 +1193,922 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
+        <v>35</v>
+      </c>
+      <c r="B27">
+        <v>256</v>
+      </c>
+      <c r="C27">
+        <v>330</v>
+      </c>
+      <c r="D27" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="28" ht="18.75" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B28" s="4"/>
+      <c r="D28" t="s">
         <v>37</v>
-      </c>
-      <c r="B27">
-        <v>285</v>
-      </c>
-      <c r="C27">
-        <v>400</v>
-      </c>
-      <c r="D27" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>38</v>
-      </c>
-      <c r="B28">
-        <v>210</v>
-      </c>
-      <c r="C28">
-        <v>300</v>
-      </c>
-      <c r="D28" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
+        <v>38</v>
+      </c>
+      <c r="C29" t="s">
         <v>39</v>
       </c>
-      <c r="B29">
-        <v>231</v>
-      </c>
-      <c r="C29">
-        <v>300</v>
-      </c>
       <c r="D29" t="s">
-        <v>5</v>
+        <v>40</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
+        <v>16</v>
+      </c>
+      <c r="C30">
+        <v>800</v>
+      </c>
+      <c r="D30" t="s">
         <v>40</v>
-      </c>
-      <c r="B30">
-        <v>200</v>
-      </c>
-      <c r="C30">
-        <v>300</v>
-      </c>
-      <c r="D30" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>41</v>
       </c>
-      <c r="B31">
-        <v>95</v>
-      </c>
       <c r="C31">
-        <v>160</v>
+        <v>1100</v>
       </c>
       <c r="D31" t="s">
-        <v>5</v>
+        <v>40</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>42</v>
+        <v>4</v>
       </c>
       <c r="B32">
-        <v>256</v>
+        <v>580</v>
       </c>
       <c r="C32">
-        <v>330</v>
+        <v>850</v>
       </c>
       <c r="D32" t="s">
-        <v>5</v>
+        <v>40</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>43</v>
-      </c>
-      <c r="B33">
-        <v>256</v>
+        <v>10</v>
       </c>
       <c r="C33">
-        <v>330</v>
+        <v>850</v>
       </c>
       <c r="D33" t="s">
-        <v>5</v>
+        <v>40</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>44</v>
-      </c>
-      <c r="B34">
-        <v>256</v>
+        <v>22</v>
       </c>
       <c r="C34">
-        <v>330</v>
+        <v>500</v>
       </c>
       <c r="D34" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="35" ht="18.75" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="B35" s="4"/>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>23</v>
+      </c>
+      <c r="C35" t="s">
+        <v>42</v>
+      </c>
       <c r="D35" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>47</v>
-      </c>
-      <c r="C36" t="s">
-        <v>48</v>
+        <v>43</v>
+      </c>
+      <c r="B36">
+        <v>575</v>
+      </c>
+      <c r="C36">
+        <v>800</v>
       </c>
       <c r="D36" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="C37">
         <v>800</v>
       </c>
       <c r="D37" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>50</v>
-      </c>
-      <c r="C38">
-        <v>1100</v>
-      </c>
+        <v>46</v>
+      </c>
+    </row>
+    <row r="38" ht="22.5" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B38" s="3"/>
       <c r="D38" t="s">
-        <v>49</v>
+        <v>37</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>4</v>
+        <v>34</v>
       </c>
       <c r="B39">
-        <v>580</v>
+        <v>703</v>
       </c>
       <c r="C39">
-        <v>850</v>
+        <v>1000</v>
       </c>
       <c r="D39" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>14</v>
+        <v>33</v>
+      </c>
+      <c r="B40">
+        <v>703</v>
       </c>
       <c r="C40">
-        <v>850</v>
+        <v>1000</v>
       </c>
       <c r="D40" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>28</v>
-      </c>
-      <c r="C41">
-        <v>500</v>
+        <v>48</v>
+      </c>
+      <c r="B41">
+        <v>703</v>
+      </c>
+      <c r="C41" t="s">
+        <v>49</v>
       </c>
       <c r="D41" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>51</v>
+        <v>8</v>
       </c>
       <c r="C42">
-        <v>550</v>
+        <v>900</v>
       </c>
       <c r="D42" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>29</v>
+        <v>23</v>
+      </c>
+      <c r="B43">
+        <v>900</v>
       </c>
       <c r="C43" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D43" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>53</v>
-      </c>
-      <c r="B44">
-        <v>575</v>
+        <v>51</v>
       </c>
       <c r="C44">
-        <v>800</v>
+        <v>1200</v>
       </c>
       <c r="D44" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="C45">
-        <v>800</v>
+        <v>1000</v>
       </c>
       <c r="D45" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="46" ht="22.5" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="B46" s="3"/>
+        <v>46</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>20</v>
+      </c>
+      <c r="C46">
+        <v>1000</v>
+      </c>
       <c r="D46" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>43</v>
-      </c>
-      <c r="B47">
-        <v>703</v>
+        <v>53</v>
       </c>
       <c r="C47">
         <v>1000</v>
       </c>
       <c r="D47" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>42</v>
-      </c>
-      <c r="B48">
-        <v>703</v>
+        <v>54</v>
       </c>
       <c r="C48">
-        <v>1000</v>
+        <v>1600</v>
       </c>
       <c r="D48" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>58</v>
-      </c>
-      <c r="B49">
-        <v>703</v>
-      </c>
-      <c r="C49" t="s">
-        <v>59</v>
+        <v>19</v>
+      </c>
+      <c r="C49">
+        <v>1100</v>
       </c>
       <c r="D49" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="C50">
-        <v>900</v>
+        <v>1100</v>
       </c>
       <c r="D50" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>29</v>
-      </c>
-      <c r="B51">
-        <v>900</v>
-      </c>
-      <c r="C51" t="s">
-        <v>60</v>
+        <v>56</v>
+      </c>
+      <c r="C51">
+        <v>3000</v>
       </c>
       <c r="D51" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="C52">
-        <v>1200</v>
+        <v>2500</v>
       </c>
       <c r="D52" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="C53">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="D53" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>26</v>
+        <v>9</v>
+      </c>
+      <c r="B54" t="s">
+        <v>59</v>
       </c>
       <c r="C54">
-        <v>1000</v>
+        <v>1500</v>
       </c>
       <c r="D54" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>63</v>
+        <v>41</v>
+      </c>
+      <c r="B55">
+        <v>1000</v>
       </c>
       <c r="C55">
-        <v>1000</v>
+        <v>1500</v>
       </c>
       <c r="D55" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>64</v>
+        <v>4</v>
+      </c>
+      <c r="B56">
+        <v>580</v>
       </c>
       <c r="C56">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="D56" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>25</v>
+        <v>18</v>
+      </c>
+      <c r="B57">
+        <v>910</v>
       </c>
       <c r="C57">
-        <v>1100</v>
+        <v>1200</v>
       </c>
       <c r="D57" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>65</v>
+        <v>31</v>
+      </c>
+      <c r="B58">
+        <v>670</v>
       </c>
       <c r="C58">
-        <v>1100</v>
+        <v>1000</v>
       </c>
       <c r="D58" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>66</v>
+        <v>10</v>
       </c>
       <c r="C59">
-        <v>3000</v>
+        <v>1400</v>
       </c>
       <c r="D59" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>67</v>
+        <v>22</v>
       </c>
       <c r="C60">
-        <v>2500</v>
+        <v>1000</v>
       </c>
       <c r="D60" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>68</v>
-      </c>
-      <c r="C61">
-        <v>2000</v>
+        <v>27</v>
+      </c>
+      <c r="B61" t="s">
+        <v>60</v>
+      </c>
+      <c r="C61" t="s">
+        <v>61</v>
       </c>
       <c r="D61" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>13</v>
-      </c>
-      <c r="B62" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="C62">
-        <v>1500</v>
+        <v>3000</v>
       </c>
       <c r="D62" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>50</v>
-      </c>
-      <c r="B63">
-        <v>1000</v>
+        <v>63</v>
       </c>
       <c r="C63">
-        <v>1500</v>
+        <v>2500</v>
       </c>
       <c r="D63" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>4</v>
-      </c>
-      <c r="B64">
-        <v>580</v>
+        <v>64</v>
       </c>
       <c r="C64">
-        <v>1500</v>
+        <v>950</v>
       </c>
       <c r="D64" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>24</v>
-      </c>
-      <c r="B65">
-        <v>910</v>
+        <v>65</v>
       </c>
       <c r="C65">
         <v>1200</v>
       </c>
       <c r="D65" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>39</v>
-      </c>
-      <c r="B66">
-        <v>670</v>
+        <v>66</v>
       </c>
       <c r="C66">
-        <v>1000</v>
+        <v>2200</v>
       </c>
       <c r="D66" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>14</v>
+        <v>67</v>
       </c>
       <c r="C67">
-        <v>1400</v>
+        <v>1300</v>
       </c>
       <c r="D67" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>28</v>
+        <v>68</v>
       </c>
       <c r="C68">
-        <v>1000</v>
+        <v>2600</v>
       </c>
       <c r="D68" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>34</v>
-      </c>
-      <c r="B69" t="s">
-        <v>70</v>
-      </c>
-      <c r="C69" t="s">
-        <v>71</v>
+        <v>69</v>
+      </c>
+      <c r="C69">
+        <v>2250</v>
       </c>
       <c r="D69" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C70">
-        <v>3000</v>
+        <v>3500</v>
       </c>
       <c r="D70" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C71">
-        <v>2500</v>
+        <v>4000</v>
       </c>
       <c r="D71" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C72">
-        <v>950</v>
+        <v>1000</v>
       </c>
       <c r="D72" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>75</v>
+        <v>16</v>
       </c>
       <c r="C73">
-        <v>1200</v>
+        <v>1500</v>
       </c>
       <c r="D73" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>76</v>
+        <v>45</v>
       </c>
       <c r="C74">
-        <v>2200</v>
+        <v>1800</v>
       </c>
       <c r="D74" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A75" t="s">
-        <v>77</v>
-      </c>
-      <c r="C75">
-        <v>1300</v>
-      </c>
-      <c r="D75" t="s">
-        <v>56</v>
-      </c>
+        <v>46</v>
+      </c>
+    </row>
+    <row r="75" ht="22.5" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A75" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="B75" s="5"/>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>78</v>
+        <v>74</v>
+      </c>
+      <c r="B76">
+        <v>175</v>
       </c>
       <c r="C76">
-        <v>2600</v>
+        <v>250</v>
       </c>
       <c r="D76" t="s">
-        <v>56</v>
+        <v>75</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>79</v>
+        <v>76</v>
+      </c>
+      <c r="B77">
+        <v>175</v>
       </c>
       <c r="C77">
-        <v>2250</v>
+        <v>250</v>
       </c>
       <c r="D77" t="s">
-        <v>56</v>
+        <v>75</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>80</v>
+        <v>77</v>
+      </c>
+      <c r="B78">
+        <v>215</v>
       </c>
       <c r="C78">
-        <v>3500</v>
+        <v>300</v>
       </c>
       <c r="D78" t="s">
-        <v>56</v>
+        <v>75</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>81</v>
+        <v>78</v>
+      </c>
+      <c r="B79">
+        <v>198</v>
       </c>
       <c r="C79">
-        <v>4000</v>
+        <v>300</v>
       </c>
       <c r="D79" t="s">
-        <v>56</v>
+        <v>75</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>82</v>
+        <v>79</v>
+      </c>
+      <c r="B80">
+        <v>200</v>
       </c>
       <c r="C80">
-        <v>1000</v>
+        <v>300</v>
       </c>
       <c r="D80" t="s">
-        <v>56</v>
+        <v>75</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>20</v>
+        <v>80</v>
+      </c>
+      <c r="B81">
+        <v>200</v>
       </c>
       <c r="C81">
-        <v>1500</v>
+        <v>300</v>
       </c>
       <c r="D81" t="s">
-        <v>56</v>
+        <v>75</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>55</v>
+        <v>81</v>
+      </c>
+      <c r="B82">
+        <v>232</v>
       </c>
       <c r="C82">
-        <v>1800</v>
+        <v>300</v>
       </c>
       <c r="D82" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="83" ht="22.5" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A83" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="B83" s="5"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>82</v>
+      </c>
+      <c r="C83">
+        <v>300</v>
+      </c>
+      <c r="D83" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B84">
         <v>175</v>
       </c>
       <c r="C84">
-        <v>250</v>
+        <v>300</v>
       </c>
       <c r="D84" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>86</v>
-      </c>
-      <c r="B85">
-        <v>175</v>
+        <v>84</v>
       </c>
       <c r="C85">
-        <v>250</v>
+        <v>300</v>
       </c>
       <c r="D85" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>87</v>
-      </c>
-      <c r="B86">
-        <v>215</v>
+        <v>85</v>
       </c>
       <c r="C86">
-        <v>300</v>
+        <v>250</v>
       </c>
       <c r="D86" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>88</v>
-      </c>
-      <c r="B87">
-        <v>198</v>
+        <v>86</v>
       </c>
       <c r="C87">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="D87" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>89</v>
-      </c>
-      <c r="B88">
-        <v>200</v>
+        <v>87</v>
+      </c>
+      <c r="B88" t="s">
+        <v>88</v>
       </c>
       <c r="C88">
         <v>300</v>
       </c>
       <c r="D88" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
+        <v>89</v>
+      </c>
+      <c r="B89" t="s">
         <v>90</v>
       </c>
-      <c r="B89">
-        <v>200</v>
-      </c>
-      <c r="C89">
-        <v>300</v>
+      <c r="C89" t="s">
+        <v>91</v>
       </c>
       <c r="D89" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B90">
-        <v>232</v>
+        <v>215</v>
       </c>
       <c r="C90">
         <v>300</v>
       </c>
       <c r="D90" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>92</v>
+        <v>93</v>
+      </c>
+      <c r="B91">
+        <v>600</v>
       </c>
       <c r="C91">
-        <v>300</v>
+        <v>800</v>
       </c>
       <c r="D91" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B92">
-        <v>175</v>
+        <v>200</v>
       </c>
       <c r="C92">
-        <v>300</v>
+        <v>270</v>
       </c>
       <c r="D92" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>94</v>
+        <v>95</v>
+      </c>
+      <c r="B93" t="s">
+        <v>90</v>
       </c>
       <c r="C93">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="D93" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>95</v>
+        <v>96</v>
+      </c>
+      <c r="B94">
+        <v>198</v>
       </c>
       <c r="C94">
-        <v>250</v>
+        <v>270</v>
       </c>
       <c r="D94" t="s">
-        <v>85</v>
+        <v>97</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>96</v>
+        <v>77</v>
+      </c>
+      <c r="B95" t="s">
+        <v>98</v>
       </c>
       <c r="C95">
-        <v>400</v>
+        <v>270</v>
       </c>
       <c r="D95" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B96" t="s">
-        <v>98</v>
-      </c>
-      <c r="C96">
-        <v>300</v>
+        <v>100</v>
+      </c>
+      <c r="C96" t="s">
+        <v>101</v>
       </c>
       <c r="D96" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>99</v>
-      </c>
-      <c r="B97" t="s">
-        <v>100</v>
-      </c>
-      <c r="C97" t="s">
-        <v>7</v>
+        <v>81</v>
+      </c>
+      <c r="B97">
+        <v>234</v>
+      </c>
+      <c r="C97">
+        <v>270</v>
       </c>
       <c r="D97" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>101</v>
-      </c>
-      <c r="B98">
-        <v>215</v>
+        <v>102</v>
+      </c>
+      <c r="B98" t="s">
+        <v>103</v>
       </c>
       <c r="C98">
-        <v>300</v>
+        <v>270</v>
       </c>
       <c r="D98" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="99" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>102</v>
-      </c>
-      <c r="B99">
-        <v>600</v>
-      </c>
-      <c r="C99">
-        <v>800</v>
-      </c>
-      <c r="D99" t="s">
-        <v>85</v>
+        <v>104</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
+        <v>105</v>
+      </c>
+      <c r="B100" t="s">
         <v>103</v>
-      </c>
-      <c r="B100">
-        <v>200</v>
       </c>
       <c r="C100">
         <v>270</v>
       </c>
       <c r="D100" t="s">
-        <v>85</v>
+        <v>106</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>104</v>
-      </c>
-      <c r="B101" t="s">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="C101">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="D101" t="s">
-        <v>85</v>
+        <v>106</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>105</v>
-      </c>
-      <c r="B102">
-        <v>198</v>
+        <v>108</v>
+      </c>
+      <c r="B102" t="s">
+        <v>109</v>
       </c>
       <c r="C102">
-        <v>270</v>
+        <v>70</v>
       </c>
       <c r="D102" t="s">
         <v>106</v>
@@ -2152,294 +2116,194 @@
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>87</v>
+        <v>110</v>
       </c>
       <c r="B103" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="C103">
-        <v>270</v>
+        <v>50</v>
       </c>
       <c r="D103" t="s">
-        <v>85</v>
+        <v>106</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="B104" t="s">
-        <v>109</v>
-      </c>
-      <c r="C104" t="s">
-        <v>110</v>
+        <v>113</v>
+      </c>
+      <c r="C104">
+        <v>40</v>
       </c>
       <c r="D104" t="s">
-        <v>85</v>
+        <v>106</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>91</v>
-      </c>
-      <c r="B105">
-        <v>234</v>
+        <v>114</v>
+      </c>
+      <c r="B105" t="s">
+        <v>115</v>
       </c>
       <c r="C105">
-        <v>270</v>
+        <v>30</v>
       </c>
       <c r="D105" t="s">
-        <v>85</v>
+        <v>106</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>111</v>
-      </c>
-      <c r="B106" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="C106">
-        <v>270</v>
+        <v>180</v>
       </c>
       <c r="D106" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="107" spans="1:1" x14ac:dyDescent="0.25">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>113</v>
+        <v>117</v>
+      </c>
+      <c r="C107">
+        <v>150</v>
+      </c>
+      <c r="D107" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>114</v>
-      </c>
-      <c r="B108" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="C108">
-        <v>270</v>
+        <v>200</v>
       </c>
       <c r="D108" t="s">
-        <v>115</v>
+        <v>106</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C109">
-        <v>300</v>
+        <v>80</v>
       </c>
       <c r="D109" t="s">
-        <v>115</v>
+        <v>106</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>117</v>
-      </c>
-      <c r="B110" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C110">
-        <v>70</v>
+        <v>160</v>
       </c>
       <c r="D110" t="s">
-        <v>115</v>
+        <v>106</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B111" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C111">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="D111" t="s">
-        <v>115</v>
+        <v>106</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B112" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C112">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="D112" t="s">
-        <v>115</v>
+        <v>106</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>123</v>
-      </c>
-      <c r="B113" t="s">
-        <v>124</v>
+        <v>125</v>
+      </c>
+      <c r="B113">
+        <v>60</v>
       </c>
       <c r="C113">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="D113" t="s">
-        <v>115</v>
+        <v>106</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>125</v>
+        <v>126</v>
+      </c>
+      <c r="B114" t="s">
+        <v>127</v>
       </c>
       <c r="C114">
-        <v>180</v>
+        <v>70</v>
       </c>
       <c r="D114" t="s">
-        <v>115</v>
+        <v>106</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C115">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="D115" t="s">
-        <v>115</v>
+        <v>106</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>127</v>
+        <v>129</v>
+      </c>
+      <c r="B116" t="s">
+        <v>130</v>
       </c>
       <c r="C116">
-        <v>200</v>
+        <v>30</v>
       </c>
       <c r="D116" t="s">
-        <v>115</v>
+        <v>106</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>128</v>
+        <v>131</v>
+      </c>
+      <c r="B117" t="s">
+        <v>115</v>
       </c>
       <c r="C117">
-        <v>80</v>
+        <v>50</v>
       </c>
       <c r="D117" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A118" t="s">
-        <v>129</v>
-      </c>
-      <c r="C118">
-        <v>160</v>
-      </c>
-      <c r="D118" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A119" t="s">
-        <v>130</v>
-      </c>
-      <c r="B119" t="s">
-        <v>131</v>
-      </c>
-      <c r="C119">
-        <v>70</v>
-      </c>
-      <c r="D119" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A120" t="s">
-        <v>132</v>
-      </c>
-      <c r="B120" t="s">
-        <v>133</v>
-      </c>
-      <c r="C120">
-        <v>100</v>
-      </c>
-      <c r="D120" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A121" t="s">
-        <v>134</v>
-      </c>
-      <c r="B121">
-        <v>60</v>
-      </c>
-      <c r="C121">
-        <v>50</v>
-      </c>
-      <c r="D121" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A122" t="s">
-        <v>135</v>
-      </c>
-      <c r="B122" t="s">
-        <v>136</v>
-      </c>
-      <c r="C122">
-        <v>70</v>
-      </c>
-      <c r="D122" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A123" t="s">
-        <v>137</v>
-      </c>
-      <c r="C123">
-        <v>100</v>
-      </c>
-      <c r="D123" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A124" t="s">
-        <v>138</v>
-      </c>
-      <c r="B124" t="s">
-        <v>139</v>
-      </c>
-      <c r="C124">
-        <v>30</v>
-      </c>
-      <c r="D124" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A125" t="s">
-        <v>140</v>
-      </c>
-      <c r="B125" t="s">
-        <v>124</v>
-      </c>
-      <c r="C125">
-        <v>50</v>
-      </c>
-      <c r="D125" t="s">
-        <v>115</v>
+        <v>106</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Order daily sales products by price-list row; drop hardcoded order list; show all price-list categories
</commit_message>
<xml_diff>
--- a/price list.xlsx
+++ b/price list.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="136">
   <si>
     <t>Product</t>
   </si>
@@ -142,6 +142,12 @@
     <t>Black&amp;white</t>
   </si>
   <si>
+    <t>320</t>
+  </si>
+  <si>
+    <t>412</t>
+  </si>
+  <si>
     <t>650</t>
   </si>
   <si>
@@ -175,6 +181,9 @@
     <t>Kenya king</t>
   </si>
   <si>
+    <t>610</t>
+  </si>
+  <si>
     <t>Chrome Gin</t>
   </si>
   <si>
@@ -302,6 +311,9 @@
   </si>
   <si>
     <t>Heineken</t>
+  </si>
+  <si>
+    <t>300</t>
   </si>
   <si>
     <t>Tusker Bottle</t>
@@ -1276,6 +1288,9 @@
       <c r="A34" t="s">
         <v>22</v>
       </c>
+      <c r="B34" t="s">
+        <v>42</v>
+      </c>
       <c r="C34">
         <v>500</v>
       </c>
@@ -1287,8 +1302,11 @@
       <c r="A35" t="s">
         <v>23</v>
       </c>
+      <c r="B35" t="s">
+        <v>43</v>
+      </c>
       <c r="C35" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D35" t="s">
         <v>40</v>
@@ -1296,7 +1314,7 @@
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B36">
         <v>575</v>
@@ -1305,23 +1323,23 @@
         <v>800</v>
       </c>
       <c r="D36" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C37">
         <v>800</v>
       </c>
       <c r="D37" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="38" ht="22.5" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B38" s="3"/>
       <c r="D38" t="s">
@@ -1339,7 +1357,7 @@
         <v>1000</v>
       </c>
       <c r="D39" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
@@ -1353,21 +1371,21 @@
         <v>1000</v>
       </c>
       <c r="D40" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B41">
         <v>703</v>
       </c>
       <c r="C41" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D41" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
@@ -1378,7 +1396,7 @@
         <v>900</v>
       </c>
       <c r="D42" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
@@ -1389,65 +1407,71 @@
         <v>900</v>
       </c>
       <c r="C43" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D43" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C44">
         <v>1200</v>
       </c>
       <c r="D44" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C45">
         <v>1000</v>
       </c>
       <c r="D45" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>20</v>
       </c>
+      <c r="B46" t="s">
+        <v>55</v>
+      </c>
       <c r="C46">
         <v>1000</v>
       </c>
       <c r="D46" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>53</v>
+        <v>56</v>
+      </c>
+      <c r="B47" t="s">
+        <v>55</v>
       </c>
       <c r="C47">
         <v>1000</v>
       </c>
       <c r="D47" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="C48">
         <v>1600</v>
       </c>
       <c r="D48" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
@@ -1458,51 +1482,51 @@
         <v>1100</v>
       </c>
       <c r="D49" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C50">
         <v>1100</v>
       </c>
       <c r="D50" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="C51">
         <v>3000</v>
       </c>
       <c r="D51" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C52">
         <v>2500</v>
       </c>
       <c r="D52" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C53">
         <v>2000</v>
       </c>
       <c r="D53" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
@@ -1510,13 +1534,13 @@
         <v>9</v>
       </c>
       <c r="B54" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C54">
         <v>1500</v>
       </c>
       <c r="D54" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
@@ -1530,7 +1554,7 @@
         <v>1500</v>
       </c>
       <c r="D55" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
@@ -1544,7 +1568,7 @@
         <v>1500</v>
       </c>
       <c r="D56" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
@@ -1558,7 +1582,7 @@
         <v>1200</v>
       </c>
       <c r="D57" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
@@ -1572,7 +1596,7 @@
         <v>1000</v>
       </c>
       <c r="D58" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
@@ -1583,7 +1607,7 @@
         <v>1400</v>
       </c>
       <c r="D59" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
@@ -1594,7 +1618,7 @@
         <v>1000</v>
       </c>
       <c r="D60" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
@@ -1602,134 +1626,134 @@
         <v>27</v>
       </c>
       <c r="B61" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C61" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="D61" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C62">
         <v>3000</v>
       </c>
       <c r="D62" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="C63">
         <v>2500</v>
       </c>
       <c r="D63" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="C64">
         <v>950</v>
       </c>
       <c r="D64" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="C65">
         <v>1200</v>
       </c>
       <c r="D65" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C66">
         <v>2200</v>
       </c>
       <c r="D66" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C67">
         <v>1300</v>
       </c>
       <c r="D67" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="C68">
         <v>2600</v>
       </c>
       <c r="D68" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C69">
         <v>2250</v>
       </c>
       <c r="D69" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="C70">
         <v>3500</v>
       </c>
       <c r="D70" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="C71">
         <v>4000</v>
       </c>
       <c r="D71" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C72">
         <v>1000</v>
       </c>
       <c r="D72" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
@@ -1740,29 +1764,29 @@
         <v>1500</v>
       </c>
       <c r="D73" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C74">
         <v>1800</v>
       </c>
       <c r="D74" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="75" ht="22.5" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A75" s="5" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B75" s="5"/>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B76">
         <v>175</v>
@@ -1771,12 +1795,12 @@
         <v>250</v>
       </c>
       <c r="D76" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="B77">
         <v>175</v>
@@ -1785,12 +1809,12 @@
         <v>250</v>
       </c>
       <c r="D77" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="B78">
         <v>215</v>
@@ -1799,12 +1823,12 @@
         <v>300</v>
       </c>
       <c r="D78" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="B79">
         <v>198</v>
@@ -1813,12 +1837,12 @@
         <v>300</v>
       </c>
       <c r="D79" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B80">
         <v>200</v>
@@ -1827,12 +1851,12 @@
         <v>300</v>
       </c>
       <c r="D80" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B81">
         <v>200</v>
@@ -1841,12 +1865,12 @@
         <v>300</v>
       </c>
       <c r="D81" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B82">
         <v>232</v>
@@ -1855,23 +1879,23 @@
         <v>300</v>
       </c>
       <c r="D82" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="C83">
         <v>300</v>
       </c>
       <c r="D83" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B84">
         <v>175</v>
@@ -1880,73 +1904,73 @@
         <v>300</v>
       </c>
       <c r="D84" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="C85">
         <v>300</v>
       </c>
       <c r="D85" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="C86">
         <v>250</v>
       </c>
       <c r="D86" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="C87">
         <v>400</v>
       </c>
       <c r="D87" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B88" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="C88">
         <v>300</v>
       </c>
       <c r="D88" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="B89" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="C89" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="D89" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="B90">
         <v>215</v>
@@ -1955,12 +1979,12 @@
         <v>300</v>
       </c>
       <c r="D90" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="B91">
         <v>600</v>
@@ -1969,12 +1993,12 @@
         <v>800</v>
       </c>
       <c r="D91" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="B92">
         <v>200</v>
@@ -1983,26 +2007,26 @@
         <v>270</v>
       </c>
       <c r="D92" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="B93" t="s">
-        <v>90</v>
-      </c>
-      <c r="C93">
-        <v>400</v>
+        <v>93</v>
+      </c>
+      <c r="C93" t="s">
+        <v>99</v>
       </c>
       <c r="D93" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="B94">
         <v>198</v>
@@ -2011,40 +2035,40 @@
         <v>270</v>
       </c>
       <c r="D94" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="B95" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="C95">
         <v>270</v>
       </c>
       <c r="D95" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="B96" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C96" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="D96" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B97">
         <v>234</v>
@@ -2053,195 +2077,195 @@
         <v>270</v>
       </c>
       <c r="D97" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="B98" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="C98">
         <v>270</v>
       </c>
       <c r="D98" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="99" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="B100" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="C100">
         <v>270</v>
       </c>
       <c r="D100" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="C101">
         <v>300</v>
       </c>
       <c r="D101" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="B102" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="C102">
         <v>70</v>
       </c>
       <c r="D102" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="B103" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="C103">
         <v>50</v>
       </c>
       <c r="D103" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="B104" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="C104">
         <v>40</v>
       </c>
       <c r="D104" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="B105" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="C105">
         <v>30</v>
       </c>
       <c r="D105" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="C106">
         <v>180</v>
       </c>
       <c r="D106" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="C107">
         <v>150</v>
       </c>
       <c r="D107" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="C108">
         <v>200</v>
       </c>
       <c r="D108" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="C109">
         <v>80</v>
       </c>
       <c r="D109" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="C110">
         <v>160</v>
       </c>
       <c r="D110" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="B111" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="C111">
         <v>70</v>
       </c>
       <c r="D111" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="B112" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="C112">
         <v>100</v>
       </c>
       <c r="D112" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="B113">
         <v>60</v>
@@ -2250,60 +2274,60 @@
         <v>50</v>
       </c>
       <c r="D113" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="B114" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="C114">
         <v>70</v>
       </c>
       <c r="D114" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="C115">
         <v>100</v>
       </c>
       <c r="D115" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="B116" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="C116">
         <v>30</v>
       </c>
       <c r="D116" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="B117" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="C117">
         <v>50</v>
       </c>
       <c r="D117" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add shop profits by date range to dashboard with Excel export; update stock sheet from price list
</commit_message>
<xml_diff>
--- a/price list.xlsx
+++ b/price list.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="139">
   <si>
     <t>Product</t>
   </si>
@@ -40,6 +40,9 @@
     <t>95</t>
   </si>
   <si>
+    <t>200</t>
+  </si>
+  <si>
     <t>V&amp;A</t>
   </si>
   <si>
@@ -94,9 +97,6 @@
     <t>Dallas</t>
   </si>
   <si>
-    <t>200</t>
-  </si>
-  <si>
     <t>General Meakings</t>
   </si>
   <si>
@@ -358,6 +358,9 @@
     <t>63</t>
   </si>
   <si>
+    <t>80</t>
+  </si>
+  <si>
     <t>Soda 350ml</t>
   </si>
   <si>
@@ -404,6 +407,12 @@
   </si>
   <si>
     <t>Lemonade</t>
+  </si>
+  <si>
+    <t>43</t>
+  </si>
+  <si>
+    <t>60</t>
   </si>
   <si>
     <t>predator</t>
@@ -874,8 +883,8 @@
       <c r="B3" t="s">
         <v>7</v>
       </c>
-      <c r="C3">
-        <v>160</v>
+      <c r="C3" t="s">
+        <v>8</v>
       </c>
       <c r="D3" t="s">
         <v>5</v>
@@ -883,7 +892,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B4">
         <v>295</v>
@@ -897,7 +906,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B5">
         <v>395</v>
@@ -911,10 +920,10 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C6">
         <v>500</v>
@@ -925,7 +934,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B7">
         <v>195</v>
@@ -939,10 +948,10 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B8" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C8">
         <v>300</v>
@@ -953,7 +962,7 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B9">
         <v>225</v>
@@ -967,10 +976,10 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B10" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C10">
         <v>550</v>
@@ -981,7 +990,7 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B11">
         <v>334</v>
@@ -995,7 +1004,7 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B12">
         <v>232</v>
@@ -1009,7 +1018,7 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B13">
         <v>208</v>
@@ -1023,7 +1032,7 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B14">
         <v>197</v>
@@ -1037,7 +1046,7 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B15">
         <v>225</v>
@@ -1051,7 +1060,7 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B16">
         <v>285</v>
@@ -1065,7 +1074,7 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B17">
         <v>200</v>
@@ -1079,13 +1088,13 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B18" t="s">
         <v>7</v>
       </c>
       <c r="C18" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="D18" t="s">
         <v>5</v>
@@ -1239,7 +1248,7 @@
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C30">
         <v>800</v>
@@ -1275,7 +1284,7 @@
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C33">
         <v>850</v>
@@ -1286,7 +1295,7 @@
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B34" t="s">
         <v>42</v>
@@ -1300,7 +1309,7 @@
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B35" t="s">
         <v>43</v>
@@ -1390,7 +1399,7 @@
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C42">
         <v>900</v>
@@ -1401,7 +1410,7 @@
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B43">
         <v>900</v>
@@ -1437,7 +1446,7 @@
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B46" t="s">
         <v>55</v>
@@ -1476,7 +1485,7 @@
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C49">
         <v>1100</v>
@@ -1531,7 +1540,7 @@
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B54" t="s">
         <v>62</v>
@@ -1573,7 +1582,7 @@
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B57">
         <v>910</v>
@@ -1601,7 +1610,7 @@
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C59">
         <v>1400</v>
@@ -1612,7 +1621,7 @@
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C60">
         <v>1000</v>
@@ -1758,7 +1767,7 @@
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C73">
         <v>1500</v>
@@ -2131,8 +2140,8 @@
       <c r="B102" t="s">
         <v>113</v>
       </c>
-      <c r="C102">
-        <v>70</v>
+      <c r="C102" t="s">
+        <v>114</v>
       </c>
       <c r="D102" t="s">
         <v>110</v>
@@ -2140,10 +2149,10 @@
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B103" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C103">
         <v>50</v>
@@ -2154,10 +2163,10 @@
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B104" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C104">
         <v>40</v>
@@ -2168,10 +2177,10 @@
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B105" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C105">
         <v>30</v>
@@ -2182,7 +2191,7 @@
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C106">
         <v>180</v>
@@ -2193,7 +2202,7 @@
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C107">
         <v>150</v>
@@ -2204,7 +2213,7 @@
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C108">
         <v>200</v>
@@ -2215,7 +2224,7 @@
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C109">
         <v>80</v>
@@ -2226,7 +2235,7 @@
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C110">
         <v>160</v>
@@ -2237,10 +2246,10 @@
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B111" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C111">
         <v>70</v>
@@ -2251,10 +2260,10 @@
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B112" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C112">
         <v>100</v>
@@ -2265,13 +2274,13 @@
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>129</v>
-      </c>
-      <c r="B113">
-        <v>60</v>
-      </c>
-      <c r="C113">
-        <v>50</v>
+        <v>130</v>
+      </c>
+      <c r="B113" t="s">
+        <v>131</v>
+      </c>
+      <c r="C113" t="s">
+        <v>132</v>
       </c>
       <c r="D113" t="s">
         <v>110</v>
@@ -2279,10 +2288,10 @@
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="B114" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="C114">
         <v>70</v>
@@ -2293,7 +2302,7 @@
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="C115">
         <v>100</v>
@@ -2304,10 +2313,10 @@
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="B116" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C116">
         <v>30</v>
@@ -2318,10 +2327,10 @@
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="B117" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C117">
         <v>50</v>

</xml_diff>